<commit_message>
Changed true values to prediction for corroded in visualisation of results
</commit_message>
<xml_diff>
--- a/results/prediction.xlsx
+++ b/results/prediction.xlsx
@@ -81046,37 +81046,37 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>10.18745440710478</v>
+        <v>7.164190769195557</v>
       </c>
       <c r="B2">
-        <v>10.93465339837988</v>
+        <v>8.11076545715332</v>
       </c>
       <c r="C2">
-        <v>7.9583826192076</v>
+        <v>7.481522083282471</v>
       </c>
       <c r="D2">
-        <v>2.795710782517715</v>
+        <v>3.524406433105469</v>
       </c>
       <c r="E2">
-        <v>5.790639450837751</v>
+        <v>5.463413715362549</v>
       </c>
       <c r="F2">
-        <v>6.115184954317368</v>
+        <v>6.175883769989014</v>
       </c>
       <c r="G2">
-        <v>8.043052625725712</v>
+        <v>8.765786170959473</v>
       </c>
       <c r="H2">
-        <v>11.86266955709876</v>
+        <v>12.24476623535156</v>
       </c>
       <c r="I2">
-        <v>11.98895258526435</v>
+        <v>8.989300727844238</v>
       </c>
       <c r="J2">
-        <v>12.29414965619717</v>
+        <v>9.413021087646484</v>
       </c>
       <c r="K2">
-        <v>13.29741225559913</v>
+        <v>10.52413368225098</v>
       </c>
       <c r="L2" t="s">
         <v>222</v>
@@ -81084,37 +81084,37 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>10.24316892009829</v>
+        <v>7.146883964538574</v>
       </c>
       <c r="B3">
-        <v>10.78583075236718</v>
+        <v>8.094620704650879</v>
       </c>
       <c r="C3">
-        <v>7.862625479995031</v>
+        <v>7.443587779998779</v>
       </c>
       <c r="D3">
-        <v>2.759343495489761</v>
+        <v>3.489659070968628</v>
       </c>
       <c r="E3">
-        <v>5.514771996825542</v>
+        <v>5.46022367477417</v>
       </c>
       <c r="F3">
-        <v>5.912619308456659</v>
+        <v>6.187378406524658</v>
       </c>
       <c r="G3">
-        <v>7.90911312120611</v>
+        <v>8.687471389770508</v>
       </c>
       <c r="H3">
-        <v>11.82564886981232</v>
+        <v>12.21590900421143</v>
       </c>
       <c r="I3">
-        <v>11.92606475771927</v>
+        <v>8.958551406860352</v>
       </c>
       <c r="J3">
-        <v>12.24183117512128</v>
+        <v>9.415287017822266</v>
       </c>
       <c r="K3">
-        <v>13.26661185932287</v>
+        <v>10.52566909790039</v>
       </c>
       <c r="L3" t="s">
         <v>222</v>
@@ -81122,37 +81122,37 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>10.12088128527995</v>
+        <v>7.0884108543396</v>
       </c>
       <c r="B4">
-        <v>10.88739539931131</v>
+        <v>8.145119667053223</v>
       </c>
       <c r="C4">
-        <v>7.84971375760487</v>
+        <v>7.605353832244873</v>
       </c>
       <c r="D4">
-        <v>2.641561709832596</v>
+        <v>3.634537696838379</v>
       </c>
       <c r="E4">
-        <v>6.308907676831817</v>
+        <v>5.36448335647583</v>
       </c>
       <c r="F4">
-        <v>5.72661357569898</v>
+        <v>6.308071136474609</v>
       </c>
       <c r="G4">
-        <v>8.287795568546978</v>
+        <v>9.03565788269043</v>
       </c>
       <c r="H4">
-        <v>11.78659650623861</v>
+        <v>12.31299114227295</v>
       </c>
       <c r="I4">
-        <v>11.7213839404357</v>
+        <v>9.123228073120117</v>
       </c>
       <c r="J4">
-        <v>12.25646470217496</v>
+        <v>9.437862396240234</v>
       </c>
       <c r="K4">
-        <v>13.2233483342515</v>
+        <v>10.52129173278809</v>
       </c>
       <c r="L4" t="s">
         <v>222</v>
@@ -81160,37 +81160,37 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>10.13948150266607</v>
+        <v>7.139424800872803</v>
       </c>
       <c r="B5">
-        <v>10.78583075236718</v>
+        <v>8.062492370605469</v>
       </c>
       <c r="C5">
-        <v>7.84971375760487</v>
+        <v>7.433556079864502</v>
       </c>
       <c r="D5">
-        <v>2.795710782517715</v>
+        <v>3.5173180103302</v>
       </c>
       <c r="E5">
-        <v>5.642694703936202</v>
+        <v>5.4779953956604</v>
       </c>
       <c r="F5">
-        <v>5.865560463058238</v>
+        <v>6.176802635192871</v>
       </c>
       <c r="G5">
-        <v>8.229609869644003</v>
+        <v>8.726306915283203</v>
       </c>
       <c r="H5">
-        <v>11.75385130328258</v>
+        <v>12.19885921478271</v>
       </c>
       <c r="I5">
-        <v>11.81088784600476</v>
+        <v>8.957883834838867</v>
       </c>
       <c r="J5">
-        <v>12.21966320902617</v>
+        <v>9.407243728637695</v>
       </c>
       <c r="K5">
-        <v>13.21839450998701</v>
+        <v>10.50785827636719</v>
       </c>
       <c r="L5" t="s">
         <v>222</v>
@@ -81198,37 +81198,37 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>10.08955209560892</v>
+        <v>7.134999752044678</v>
       </c>
       <c r="B6">
-        <v>10.67918710431254</v>
+        <v>8.060457229614258</v>
       </c>
       <c r="C6">
-        <v>7.824712468723903</v>
+        <v>7.410646438598633</v>
       </c>
       <c r="D6">
-        <v>2.721603552122224</v>
+        <v>3.487688302993774</v>
       </c>
       <c r="E6">
-        <v>5.530310445033498</v>
+        <v>5.486449718475342</v>
       </c>
       <c r="F6">
-        <v>5.778481700556402</v>
+        <v>6.173127174377441</v>
       </c>
       <c r="G6">
-        <v>8.190676161323875</v>
+        <v>8.683982849121094</v>
       </c>
       <c r="H6">
-        <v>11.72681208035344</v>
+        <v>12.19118213653564</v>
       </c>
       <c r="I6">
-        <v>11.75447633333297</v>
+        <v>8.939350128173828</v>
       </c>
       <c r="J6">
-        <v>12.16602003204375</v>
+        <v>9.40318489074707</v>
       </c>
       <c r="K6">
-        <v>13.15592064695505</v>
+        <v>10.50686645507812</v>
       </c>
       <c r="L6" t="s">
         <v>222</v>
@@ -81236,37 +81236,37 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>10.09369460360407</v>
+        <v>7.069802761077881</v>
       </c>
       <c r="B7">
-        <v>10.75856459787929</v>
+        <v>8.087602615356445</v>
       </c>
       <c r="C7">
-        <v>7.803616502311114</v>
+        <v>7.428328037261963</v>
       </c>
       <c r="D7">
-        <v>2.759343495489761</v>
+        <v>3.485660314559937</v>
       </c>
       <c r="E7">
-        <v>5.028984578218987</v>
+        <v>5.425857067108154</v>
       </c>
       <c r="F7">
-        <v>5.526936019747212</v>
+        <v>6.232194900512695</v>
       </c>
       <c r="G7">
-        <v>8.103471860975706</v>
+        <v>8.623250961303711</v>
       </c>
       <c r="H7">
-        <v>11.67339329239558</v>
+        <v>12.20251941680908</v>
       </c>
       <c r="I7">
-        <v>11.81689090585536</v>
+        <v>8.944780349731445</v>
       </c>
       <c r="J7">
-        <v>12.0854919494438</v>
+        <v>9.400962829589844</v>
       </c>
       <c r="K7">
-        <v>13.13680744578279</v>
+        <v>10.50839614868164</v>
       </c>
       <c r="L7" t="s">
         <v>222</v>
@@ -81274,37 +81274,37 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>10.06622032916697</v>
+        <v>7.128314971923828</v>
       </c>
       <c r="B8">
-        <v>10.69088373641538</v>
+        <v>8.051462173461914</v>
       </c>
       <c r="C8">
-        <v>7.842758711064346</v>
+        <v>7.361822605133057</v>
       </c>
       <c r="D8">
-        <v>2.682383254353312</v>
+        <v>3.419692039489746</v>
       </c>
       <c r="E8">
-        <v>5.485257823115336</v>
+        <v>5.494924545288086</v>
       </c>
       <c r="F8">
-        <v>5.788540022831065</v>
+        <v>6.137596607208252</v>
       </c>
       <c r="G8">
-        <v>8.23649900229349</v>
+        <v>8.596458435058594</v>
       </c>
       <c r="H8">
-        <v>11.61459818897559</v>
+        <v>12.15928745269775</v>
       </c>
       <c r="I8">
-        <v>11.8300045134636</v>
+        <v>8.895545959472656</v>
       </c>
       <c r="J8">
-        <v>12.11373194196401</v>
+        <v>9.376971244812012</v>
       </c>
       <c r="K8">
-        <v>13.12535224030023</v>
+        <v>10.48973655700684</v>
       </c>
       <c r="L8" t="s">
         <v>222</v>
@@ -81312,37 +81312,37 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>9.957607393474596</v>
+        <v>7.113456249237061</v>
       </c>
       <c r="B9">
-        <v>10.59240356933425</v>
+        <v>8.061090469360352</v>
       </c>
       <c r="C9">
-        <v>7.703509181989499</v>
+        <v>7.398766994476318</v>
       </c>
       <c r="D9">
-        <v>2.682383254353312</v>
+        <v>3.464852571487427</v>
       </c>
       <c r="E9">
-        <v>5.275844482286887</v>
+        <v>5.483791351318359</v>
       </c>
       <c r="F9">
-        <v>5.618789166946144</v>
+        <v>6.18822193145752</v>
       </c>
       <c r="G9">
-        <v>8.06618817134161</v>
+        <v>8.651357650756836</v>
       </c>
       <c r="H9">
-        <v>11.56966175253297</v>
+        <v>12.18665885925293</v>
       </c>
       <c r="I9">
-        <v>11.68294949114163</v>
+        <v>8.92951774597168</v>
       </c>
       <c r="J9">
-        <v>11.99441153049895</v>
+        <v>9.39967155456543</v>
       </c>
       <c r="K9">
-        <v>13.05507619254936</v>
+        <v>10.50749206542969</v>
       </c>
       <c r="L9" t="s">
         <v>222</v>
@@ -81350,37 +81350,37 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>10.00839795690907</v>
+        <v>7.074497222900391</v>
       </c>
       <c r="B10">
-        <v>10.56640459731058</v>
+        <v>8.079272270202637</v>
       </c>
       <c r="C10">
-        <v>7.846676870225138</v>
+        <v>7.422913074493408</v>
       </c>
       <c r="D10">
-        <v>2.795710782517715</v>
+        <v>3.470289468765259</v>
       </c>
       <c r="E10">
-        <v>4.965173036298562</v>
+        <v>5.426188945770264</v>
       </c>
       <c r="F10">
-        <v>5.519105204169787</v>
+        <v>6.208460807800293</v>
       </c>
       <c r="G10">
-        <v>8.139415297032262</v>
+        <v>8.603778839111328</v>
       </c>
       <c r="H10">
-        <v>11.53531081103786</v>
+        <v>12.19498729705811</v>
       </c>
       <c r="I10">
-        <v>11.9751209145677</v>
+        <v>8.932440757751465</v>
       </c>
       <c r="J10">
-        <v>12.06196488550392</v>
+        <v>9.396138191223145</v>
       </c>
       <c r="K10">
-        <v>13.07780059903511</v>
+        <v>10.50826072692871</v>
       </c>
       <c r="L10" t="s">
         <v>222</v>
@@ -81388,37 +81388,37 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>10.01537672009158</v>
+        <v>7.210177898406982</v>
       </c>
       <c r="B11">
-        <v>10.5391233040124</v>
+        <v>7.983603000640869</v>
       </c>
       <c r="C11">
-        <v>7.815789781801988</v>
+        <v>7.252441883087158</v>
       </c>
       <c r="D11">
-        <v>2.353878387381596</v>
+        <v>3.256672620773315</v>
       </c>
       <c r="E11">
-        <v>5.787238120854426</v>
+        <v>5.532107830047607</v>
       </c>
       <c r="F11">
-        <v>5.753920376344398</v>
+        <v>5.976643562316895</v>
       </c>
       <c r="G11">
-        <v>8.623175733575462</v>
+        <v>8.435321807861328</v>
       </c>
       <c r="H11">
-        <v>11.50211614317996</v>
+        <v>12.04977130889893</v>
       </c>
       <c r="I11">
-        <v>11.69302232395811</v>
+        <v>8.755634307861328</v>
       </c>
       <c r="J11">
-        <v>11.98683119610423</v>
+        <v>9.327564239501953</v>
       </c>
       <c r="K11">
-        <v>13.0117719197493</v>
+        <v>10.46822166442871</v>
       </c>
       <c r="L11" t="s">
         <v>222</v>
@@ -81426,37 +81426,37 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>10.76473527387915</v>
+        <v>7.669240474700928</v>
       </c>
       <c r="B12">
-        <v>11.44838694383266</v>
+        <v>8.981767654418945</v>
       </c>
       <c r="C12">
-        <v>8.226246542695968</v>
+        <v>7.727635860443115</v>
       </c>
       <c r="D12">
-        <v>2.864703011147087</v>
+        <v>3.823773145675659</v>
       </c>
       <c r="E12">
-        <v>7.030464428060571</v>
+        <v>8.037128448486328</v>
       </c>
       <c r="F12">
-        <v>5.718917941639756</v>
+        <v>6.707357883453369</v>
       </c>
       <c r="G12">
-        <v>7.662078876803823</v>
+        <v>8.926900863647461</v>
       </c>
       <c r="H12">
-        <v>12.54132528946476</v>
+        <v>12.51622295379639</v>
       </c>
       <c r="I12">
-        <v>12.10961069218929</v>
+        <v>9.13279914855957</v>
       </c>
       <c r="J12">
-        <v>12.87520316611729</v>
+        <v>9.696168899536133</v>
       </c>
       <c r="K12">
-        <v>13.76344386563425</v>
+        <v>10.94185447692871</v>
       </c>
       <c r="L12" t="s">
         <v>223</v>
@@ -81464,37 +81464,37 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>10.76049997341059</v>
+        <v>7.719478607177734</v>
       </c>
       <c r="B13">
-        <v>11.37716938241427</v>
+        <v>9.029376983642578</v>
       </c>
       <c r="C13">
-        <v>8.268731832117737</v>
+        <v>7.765392303466797</v>
       </c>
       <c r="D13">
-        <v>2.721603552122224</v>
+        <v>3.875698328018188</v>
       </c>
       <c r="E13">
-        <v>6.958131470459343</v>
+        <v>8.064937591552734</v>
       </c>
       <c r="F13">
-        <v>5.946344111827512</v>
+        <v>6.735772609710693</v>
       </c>
       <c r="G13">
-        <v>7.809220611253454</v>
+        <v>8.949073791503906</v>
       </c>
       <c r="H13">
-        <v>12.52012417589325</v>
+        <v>12.53979873657227</v>
       </c>
       <c r="I13">
-        <v>12.13103774698981</v>
+        <v>9.154186248779297</v>
       </c>
       <c r="J13">
-        <v>12.8758573692627</v>
+        <v>9.722973823547363</v>
       </c>
       <c r="K13">
-        <v>13.75735046625958</v>
+        <v>10.97372055053711</v>
       </c>
       <c r="L13" t="s">
         <v>223</v>
@@ -81502,37 +81502,37 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>10.7906927103786</v>
+        <v>7.603953838348389</v>
       </c>
       <c r="B14">
-        <v>11.51752597637089</v>
+        <v>8.906247138977051</v>
       </c>
       <c r="C14">
-        <v>8.190539272974506</v>
+        <v>7.716779708862305</v>
       </c>
       <c r="D14">
-        <v>3.047025567941541</v>
+        <v>3.782360315322876</v>
       </c>
       <c r="E14">
-        <v>7.013115784639963</v>
+        <v>7.963951587677002</v>
       </c>
       <c r="F14">
-        <v>5.785332281379343</v>
+        <v>6.662105083465576</v>
       </c>
       <c r="G14">
-        <v>7.859556130315068</v>
+        <v>8.929285049438477</v>
       </c>
       <c r="H14">
-        <v>12.4969967485419</v>
+        <v>12.48010540008545</v>
       </c>
       <c r="I14">
-        <v>12.08244757713283</v>
+        <v>9.111193656921387</v>
       </c>
       <c r="J14">
-        <v>12.86254719800897</v>
+        <v>9.672447204589844</v>
       </c>
       <c r="K14">
-        <v>13.72211399023589</v>
+        <v>10.9118824005127</v>
       </c>
       <c r="L14" t="s">
         <v>223</v>
@@ -81540,37 +81540,37 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>10.73615510281665</v>
+        <v>7.567496776580811</v>
       </c>
       <c r="B15">
-        <v>11.49153156887714</v>
+        <v>8.851802825927734</v>
       </c>
       <c r="C15">
-        <v>8.166216268592143</v>
+        <v>7.711580753326416</v>
       </c>
       <c r="D15">
-        <v>3.292147808583199</v>
+        <v>3.748436212539673</v>
       </c>
       <c r="E15">
-        <v>7.037808416986432</v>
+        <v>7.924636840820312</v>
       </c>
       <c r="F15">
-        <v>5.868151524957849</v>
+        <v>6.640189170837402</v>
       </c>
       <c r="G15">
-        <v>7.80116902790133</v>
+        <v>8.939108848571777</v>
       </c>
       <c r="H15">
-        <v>12.48427808116805</v>
+        <v>12.45362663269043</v>
       </c>
       <c r="I15">
-        <v>12.07563487414962</v>
+        <v>9.100736618041992</v>
       </c>
       <c r="J15">
-        <v>12.8627776947007</v>
+        <v>9.664119720458984</v>
       </c>
       <c r="K15">
-        <v>13.73065322263299</v>
+        <v>10.88632965087891</v>
       </c>
       <c r="L15" t="s">
         <v>223</v>
@@ -81578,37 +81578,37 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>10.75979234983972</v>
+        <v>7.624914646148682</v>
       </c>
       <c r="B16">
-        <v>11.37116986608195</v>
+        <v>8.953777313232422</v>
       </c>
       <c r="C16">
-        <v>8.225949236318703</v>
+        <v>7.723233222961426</v>
       </c>
       <c r="D16">
-        <v>2.960015100042408</v>
+        <v>3.81092095375061</v>
       </c>
       <c r="E16">
-        <v>7.069968596785415</v>
+        <v>8.012182235717773</v>
       </c>
       <c r="F16">
-        <v>5.785332281379343</v>
+        <v>6.689337730407715</v>
       </c>
       <c r="G16">
-        <v>7.850459505023849</v>
+        <v>8.915340423583984</v>
       </c>
       <c r="H16">
-        <v>12.47393395295754</v>
+        <v>12.49600505828857</v>
       </c>
       <c r="I16">
-        <v>12.05762419620737</v>
+        <v>9.124882698059082</v>
       </c>
       <c r="J16">
-        <v>12.84967062304855</v>
+        <v>9.681763648986816</v>
       </c>
       <c r="K16">
-        <v>13.7302782037566</v>
+        <v>10.92659187316895</v>
       </c>
       <c r="L16" t="s">
         <v>223</v>
@@ -81616,37 +81616,37 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17">
-        <v>10.78357523113803</v>
+        <v>7.724518775939941</v>
       </c>
       <c r="B17">
-        <v>11.49153156887714</v>
+        <v>9.020786285400391</v>
       </c>
       <c r="C17">
-        <v>8.238947945059326</v>
+        <v>7.765933513641357</v>
       </c>
       <c r="D17">
-        <v>2.682383254353312</v>
+        <v>3.870849847793579</v>
       </c>
       <c r="E17">
-        <v>7.103413423484152</v>
+        <v>8.07813835144043</v>
       </c>
       <c r="F17">
-        <v>5.851375735140308</v>
+        <v>6.730086326599121</v>
       </c>
       <c r="G17">
-        <v>7.649810182938724</v>
+        <v>8.961858749389648</v>
       </c>
       <c r="H17">
-        <v>12.46316599173634</v>
+        <v>12.54918956756592</v>
       </c>
       <c r="I17">
-        <v>12.09723696514279</v>
+        <v>9.154519081115723</v>
       </c>
       <c r="J17">
-        <v>12.89235464708305</v>
+        <v>9.722890853881836</v>
       </c>
       <c r="K17">
-        <v>13.7518711876694</v>
+        <v>10.9782657623291</v>
       </c>
       <c r="L17" t="s">
         <v>223</v>
@@ -81654,37 +81654,37 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18">
-        <v>10.75506197680297</v>
+        <v>7.603856563568115</v>
       </c>
       <c r="B18">
-        <v>11.47308677851077</v>
+        <v>8.901908874511719</v>
       </c>
       <c r="C18">
-        <v>8.164952857187595</v>
+        <v>7.709210395812988</v>
       </c>
       <c r="D18">
-        <v>3.127067506384013</v>
+        <v>3.772567987442017</v>
       </c>
       <c r="E18">
-        <v>7.094695777024091</v>
+        <v>7.951913356781006</v>
       </c>
       <c r="F18">
-        <v>5.81889912642444</v>
+        <v>6.664803504943848</v>
       </c>
       <c r="G18">
-        <v>7.682197920653789</v>
+        <v>8.929685592651367</v>
       </c>
       <c r="H18">
-        <v>12.45300368442047</v>
+        <v>12.4765157699585</v>
       </c>
       <c r="I18">
-        <v>12.10850881766768</v>
+        <v>9.106331825256348</v>
       </c>
       <c r="J18">
-        <v>12.84519473268245</v>
+        <v>9.668970108032227</v>
       </c>
       <c r="K18">
-        <v>13.712516375885</v>
+        <v>10.90693855285645</v>
       </c>
       <c r="L18" t="s">
         <v>223</v>
@@ -81692,37 +81692,37 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19">
-        <v>10.70099474842032</v>
+        <v>7.652152538299561</v>
       </c>
       <c r="B19">
-        <v>11.35334339514576</v>
+        <v>8.977133750915527</v>
       </c>
       <c r="C19">
-        <v>8.188689124444201</v>
+        <v>7.72501802444458</v>
       </c>
       <c r="D19">
-        <v>2.960015100042408</v>
+        <v>3.822075128555298</v>
       </c>
       <c r="E19">
-        <v>7.001043233648609</v>
+        <v>8.02230167388916</v>
       </c>
       <c r="F19">
-        <v>5.813056909166414</v>
+        <v>6.709784507751465</v>
       </c>
       <c r="G19">
-        <v>7.661498009040496</v>
+        <v>8.927239418029785</v>
       </c>
       <c r="H19">
-        <v>12.44419391315152</v>
+        <v>12.50169372558594</v>
       </c>
       <c r="I19">
-        <v>12.13813873457512</v>
+        <v>9.129763603210449</v>
       </c>
       <c r="J19">
-        <v>12.81959624473754</v>
+        <v>9.688100814819336</v>
       </c>
       <c r="K19">
-        <v>13.68465368049063</v>
+        <v>10.93247222900391</v>
       </c>
       <c r="L19" t="s">
         <v>223</v>
@@ -81730,37 +81730,37 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20">
-        <v>10.71786860775271</v>
+        <v>7.598369598388672</v>
       </c>
       <c r="B20">
-        <v>11.43730353043051</v>
+        <v>8.897219657897949</v>
       </c>
       <c r="C20">
-        <v>8.169682470277342</v>
+        <v>7.709290981292725</v>
       </c>
       <c r="D20">
-        <v>3.201176962054259</v>
+        <v>3.770913362503052</v>
       </c>
       <c r="E20">
-        <v>6.995969615459113</v>
+        <v>7.948566436767578</v>
       </c>
       <c r="F20">
-        <v>5.853253651238048</v>
+        <v>6.672333717346191</v>
       </c>
       <c r="G20">
-        <v>7.618160075443261</v>
+        <v>8.932639122009277</v>
       </c>
       <c r="H20">
-        <v>12.43141976719893</v>
+        <v>12.46806526184082</v>
       </c>
       <c r="I20">
-        <v>12.13748445286399</v>
+        <v>9.106504440307617</v>
       </c>
       <c r="J20">
-        <v>12.83188331957301</v>
+        <v>9.668972015380859</v>
       </c>
       <c r="K20">
-        <v>13.70229084399968</v>
+        <v>10.9035701751709</v>
       </c>
       <c r="L20" t="s">
         <v>223</v>
@@ -81768,37 +81768,37 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21">
-        <v>10.7628551299535</v>
+        <v>7.601551532745361</v>
       </c>
       <c r="B21">
-        <v>11.49141804974853</v>
+        <v>8.891574859619141</v>
       </c>
       <c r="C21">
-        <v>8.237185303605333</v>
+        <v>7.71199369430542</v>
       </c>
       <c r="D21">
-        <v>3.17707967179902</v>
+        <v>3.772971868515015</v>
       </c>
       <c r="E21">
-        <v>7.043644994825126</v>
+        <v>7.9449143409729</v>
       </c>
       <c r="F21">
-        <v>5.868151524957849</v>
+        <v>6.654940605163574</v>
       </c>
       <c r="G21">
-        <v>7.686173628803736</v>
+        <v>8.925403594970703</v>
       </c>
       <c r="H21">
-        <v>12.41954670886316</v>
+        <v>12.4746732711792</v>
       </c>
       <c r="I21">
-        <v>12.03987375326754</v>
+        <v>9.104419708251953</v>
       </c>
       <c r="J21">
-        <v>12.89690325490988</v>
+        <v>9.669065475463867</v>
       </c>
       <c r="K21">
-        <v>13.73772797993911</v>
+        <v>10.90205192565918</v>
       </c>
       <c r="L21" t="s">
         <v>223</v>
@@ -81806,37 +81806,37 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22">
-        <v>7.471173542620601</v>
+        <v>8.415657043457031</v>
       </c>
       <c r="B22">
-        <v>8.572803095822961</v>
+        <v>8.055915832519531</v>
       </c>
       <c r="C22">
-        <v>3.340108902280432</v>
+        <v>4.914890766143799</v>
       </c>
       <c r="D22">
-        <v>1.660731206821651</v>
+        <v>5.494258880615234</v>
       </c>
       <c r="E22">
-        <v>4.567814572454688</v>
+        <v>8.493434906005859</v>
       </c>
       <c r="F22">
-        <v>3.101093377446938</v>
+        <v>4.254622936248779</v>
       </c>
       <c r="G22">
-        <v>3.699115772671582</v>
+        <v>8.811978340148926</v>
       </c>
       <c r="H22">
-        <v>7.861341795599989</v>
+        <v>8.802186965942383</v>
       </c>
       <c r="I22">
-        <v>8.3533661125464</v>
+        <v>7.640530109405518</v>
       </c>
       <c r="J22">
-        <v>10.41979811647799</v>
+        <v>9.914070129394531</v>
       </c>
       <c r="K22">
-        <v>11.67849640185174</v>
+        <v>11.87989044189453</v>
       </c>
       <c r="L22" t="s">
         <v>224</v>
@@ -81844,37 +81844,37 @@
     </row>
     <row r="23" spans="1:12">
       <c r="A23">
-        <v>7.508421423932544</v>
+        <v>8.173870086669922</v>
       </c>
       <c r="B23">
-        <v>9.00062476098201</v>
+        <v>7.825865745544434</v>
       </c>
       <c r="C23">
-        <v>3.214421920947292</v>
+        <v>4.706960201263428</v>
       </c>
       <c r="D23">
-        <v>1.660731206821651</v>
+        <v>5.59357738494873</v>
       </c>
       <c r="E23">
-        <v>3.625821170217794</v>
+        <v>7.024263858795166</v>
       </c>
       <c r="F23">
-        <v>2.975928646257311</v>
+        <v>3.990477085113525</v>
       </c>
       <c r="G23">
-        <v>4.324868220833933</v>
+        <v>8.723445892333984</v>
       </c>
       <c r="H23">
-        <v>7.755291211028034</v>
+        <v>7.801899909973145</v>
       </c>
       <c r="I23">
-        <v>8.046300206811237</v>
+        <v>7.377681732177734</v>
       </c>
       <c r="J23">
-        <v>10.64582165188132</v>
+        <v>9.52467155456543</v>
       </c>
       <c r="K23">
-        <v>12.10426137938349</v>
+        <v>11.61178779602051</v>
       </c>
       <c r="L23" t="s">
         <v>224</v>
@@ -81882,37 +81882,37 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24">
-        <v>7.696717511876821</v>
+        <v>8.173632621765137</v>
       </c>
       <c r="B24">
-        <v>8.917906226288533</v>
+        <v>7.824084281921387</v>
       </c>
       <c r="C24">
-        <v>3.735020875363745</v>
+        <v>4.604106426239014</v>
       </c>
       <c r="D24">
-        <v>1.660731206821651</v>
+        <v>5.549721717834473</v>
       </c>
       <c r="E24">
-        <v>4.13605496199352</v>
+        <v>6.99819803237915</v>
       </c>
       <c r="F24">
-        <v>3.158251203051766</v>
+        <v>3.957726955413818</v>
       </c>
       <c r="G24">
-        <v>4.557120747413707</v>
+        <v>8.74009895324707</v>
       </c>
       <c r="H24">
-        <v>7.596727079763401</v>
+        <v>7.625475883483887</v>
       </c>
       <c r="I24">
-        <v>8.13804532669038</v>
+        <v>7.274117946624756</v>
       </c>
       <c r="J24">
-        <v>10.8187777840767</v>
+        <v>9.453956604003906</v>
       </c>
       <c r="K24">
-        <v>12.35748625155753</v>
+        <v>11.56384086608887</v>
       </c>
       <c r="L24" t="s">
         <v>224</v>
@@ -81920,37 +81920,37 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25">
-        <v>7.9993056911933</v>
+        <v>8.177740097045898</v>
       </c>
       <c r="B25">
-        <v>8.616267369392309</v>
+        <v>7.789597988128662</v>
       </c>
       <c r="C25">
-        <v>3.643416498641661</v>
+        <v>4.565447807312012</v>
       </c>
       <c r="D25">
-        <v>1.660731206821651</v>
+        <v>5.544360160827637</v>
       </c>
       <c r="E25">
-        <v>3.796736725282063</v>
+        <v>6.985891342163086</v>
       </c>
       <c r="F25">
-        <v>2.906936417627939</v>
+        <v>3.933480262756348</v>
       </c>
       <c r="G25">
-        <v>4.792963780872861</v>
+        <v>8.728744506835938</v>
       </c>
       <c r="H25">
-        <v>7.541683099882111</v>
+        <v>7.581769943237305</v>
       </c>
       <c r="I25">
-        <v>8.077826462666872</v>
+        <v>7.25204610824585</v>
       </c>
       <c r="J25">
-        <v>10.66572019029683</v>
+        <v>9.382359504699707</v>
       </c>
       <c r="K25">
-        <v>12.08645041897361</v>
+        <v>11.53067398071289</v>
       </c>
       <c r="L25" t="s">
         <v>224</v>
@@ -81958,37 +81958,37 @@
     </row>
     <row r="26" spans="1:12">
       <c r="A26">
-        <v>7.46482840852831</v>
+        <v>8.094085693359375</v>
       </c>
       <c r="B26">
-        <v>8.545240560756181</v>
+        <v>7.853034019470215</v>
       </c>
       <c r="C26">
-        <v>3.613916116239239</v>
+        <v>4.631540298461914</v>
       </c>
       <c r="D26">
-        <v>1.660731206821651</v>
+        <v>5.527945995330811</v>
       </c>
       <c r="E26">
-        <v>4.350994453792913</v>
+        <v>6.941956996917725</v>
       </c>
       <c r="F26">
-        <v>3.263610718709092</v>
+        <v>3.947472095489502</v>
       </c>
       <c r="G26">
-        <v>4.388179886751139</v>
+        <v>8.625520706176758</v>
       </c>
       <c r="H26">
-        <v>7.541683099882111</v>
+        <v>7.619376182556152</v>
       </c>
       <c r="I26">
-        <v>8.197905687806001</v>
+        <v>7.210936546325684</v>
       </c>
       <c r="J26">
-        <v>10.68064393305867</v>
+        <v>9.500703811645508</v>
       </c>
       <c r="K26">
-        <v>12.20788211744799</v>
+        <v>11.49482536315918</v>
       </c>
       <c r="L26" t="s">
         <v>224</v>
@@ -81996,37 +81996,37 @@
     </row>
     <row r="27" spans="1:12">
       <c r="A27">
-        <v>7.726555776458847</v>
+        <v>8.203117370605469</v>
       </c>
       <c r="B27">
-        <v>9.055244762510167</v>
+        <v>7.780672073364258</v>
       </c>
       <c r="C27">
-        <v>3.680512044779201</v>
+        <v>4.549213886260986</v>
       </c>
       <c r="D27">
-        <v>1.766090722478977</v>
+        <v>5.509829044342041</v>
       </c>
       <c r="E27">
-        <v>4.282820061277547</v>
+        <v>7.000385761260986</v>
       </c>
       <c r="F27">
-        <v>3.381394754365976</v>
+        <v>3.944396495819092</v>
       </c>
       <c r="G27">
-        <v>4.626343333387389</v>
+        <v>8.795440673828125</v>
       </c>
       <c r="H27">
-        <v>7.469907533080029</v>
+        <v>7.55244779586792</v>
       </c>
       <c r="I27">
-        <v>8.376653066335441</v>
+        <v>7.272119045257568</v>
       </c>
       <c r="J27">
-        <v>10.80104841030859</v>
+        <v>9.390628814697266</v>
       </c>
       <c r="K27">
-        <v>12.37911984478285</v>
+        <v>11.54242897033691</v>
       </c>
       <c r="L27" t="s">
         <v>224</v>
@@ -82034,37 +82034,37 @@
     </row>
     <row r="28" spans="1:12">
       <c r="A28">
-        <v>7.90961177678691</v>
+        <v>8.191657066345215</v>
       </c>
       <c r="B28">
-        <v>8.807870822698264</v>
+        <v>7.702161312103271</v>
       </c>
       <c r="C28">
-        <v>3.328228760201859</v>
+        <v>4.540108680725098</v>
       </c>
       <c r="D28">
-        <v>1.660731206821651</v>
+        <v>5.565369129180908</v>
       </c>
       <c r="E28">
-        <v>4.181201691205007</v>
+        <v>7.058628559112549</v>
       </c>
       <c r="F28">
-        <v>2.465104022491821</v>
+        <v>3.795610904693604</v>
       </c>
       <c r="G28">
-        <v>4.349613916663858</v>
+        <v>8.792476654052734</v>
       </c>
       <c r="H28">
-        <v>7.408530566894626</v>
+        <v>7.479673385620117</v>
       </c>
       <c r="I28">
-        <v>7.2754797514151</v>
+        <v>7.296975612640381</v>
       </c>
       <c r="J28">
-        <v>10.53313271460399</v>
+        <v>9.397233963012695</v>
       </c>
       <c r="K28">
-        <v>11.90576303356477</v>
+        <v>11.5704174041748</v>
       </c>
       <c r="L28" t="s">
         <v>224</v>
@@ -82072,37 +82072,37 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29">
-        <v>7.855113965017139</v>
+        <v>9.591160774230957</v>
       </c>
       <c r="B29">
-        <v>9.090972769055933</v>
+        <v>7.62637186050415</v>
       </c>
       <c r="C29">
-        <v>4.845061507190932</v>
+        <v>7.642890930175781</v>
       </c>
       <c r="D29">
-        <v>1.660731206821651</v>
+        <v>2.523177146911621</v>
       </c>
       <c r="E29">
-        <v>3.826223257755535</v>
+        <v>10.13663673400879</v>
       </c>
       <c r="F29">
-        <v>2.75278734494282</v>
+        <v>5.58150053024292</v>
       </c>
       <c r="G29">
-        <v>4.511175695839976</v>
+        <v>9.624845504760742</v>
       </c>
       <c r="H29">
-        <v>7.392579107051412</v>
+        <v>11.98579978942871</v>
       </c>
       <c r="I29">
-        <v>8.271576755840877</v>
+        <v>8.731450080871582</v>
       </c>
       <c r="J29">
-        <v>10.67423857684958</v>
+        <v>9.962675094604492</v>
       </c>
       <c r="K29">
-        <v>12.1783359605742</v>
+        <v>11.5953311920166</v>
       </c>
       <c r="L29" t="s">
         <v>224</v>
@@ -82110,37 +82110,37 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30">
-        <v>7.623424914164102</v>
+        <v>8.097263336181641</v>
       </c>
       <c r="B30">
-        <v>8.545240560756181</v>
+        <v>7.576784133911133</v>
       </c>
       <c r="C30">
-        <v>3.393763149443016</v>
+        <v>4.454545021057129</v>
       </c>
       <c r="D30">
-        <v>1.660731206821651</v>
+        <v>5.26482105255127</v>
       </c>
       <c r="E30">
-        <v>4.150164719885462</v>
+        <v>6.87241268157959</v>
       </c>
       <c r="F30">
-        <v>2.61925327374663</v>
+        <v>3.778116703033447</v>
       </c>
       <c r="G30">
-        <v>4.396326677716558</v>
+        <v>8.611124038696289</v>
       </c>
       <c r="H30">
-        <v>7.254884810077338</v>
+        <v>7.516740798950195</v>
       </c>
       <c r="I30">
-        <v>8.204003480997784</v>
+        <v>7.165470600128174</v>
       </c>
       <c r="J30">
-        <v>10.76626028562306</v>
+        <v>9.168681144714355</v>
       </c>
       <c r="K30">
-        <v>12.31261246353755</v>
+        <v>11.23785972595215</v>
       </c>
       <c r="L30" t="s">
         <v>224</v>
@@ -82148,37 +82148,37 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31">
-        <v>7.252919629490855</v>
+        <v>8.048053741455078</v>
       </c>
       <c r="B31">
-        <v>8.672803148836982</v>
+        <v>7.480017185211182</v>
       </c>
       <c r="C31">
-        <v>3.091042453358316</v>
+        <v>4.415334701538086</v>
       </c>
       <c r="D31">
-        <v>1.660731206821651</v>
+        <v>5.202467441558838</v>
       </c>
       <c r="E31">
-        <v>3.940502584741369</v>
+        <v>6.862140655517578</v>
       </c>
       <c r="F31">
-        <v>2.465104022491821</v>
+        <v>3.650016307830811</v>
       </c>
       <c r="G31">
-        <v>4.167080296992323</v>
+        <v>8.465394973754883</v>
       </c>
       <c r="H31">
-        <v>7.254884810077338</v>
+        <v>7.443991184234619</v>
       </c>
       <c r="I31">
-        <v>7.67063559030285</v>
+        <v>7.195464611053467</v>
       </c>
       <c r="J31">
-        <v>10.24134771839494</v>
+        <v>9.135988235473633</v>
       </c>
       <c r="K31">
-        <v>11.61594323754723</v>
+        <v>11.21120643615723</v>
       </c>
       <c r="L31" t="s">
         <v>224</v>
@@ -82186,37 +82186,37 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32">
-        <v>11.22095272073729</v>
+        <v>9.026865005493164</v>
       </c>
       <c r="B32">
-        <v>11.08829452506858</v>
+        <v>9.266526222229004</v>
       </c>
       <c r="C32">
-        <v>8.717481999423201</v>
+        <v>8.729704856872559</v>
       </c>
       <c r="D32">
-        <v>5.852068018224339</v>
+        <v>6.334249973297119</v>
       </c>
       <c r="E32">
-        <v>6.70250622436576</v>
+        <v>7.714353084564209</v>
       </c>
       <c r="F32">
-        <v>7.757207673835019</v>
+        <v>8.005621910095215</v>
       </c>
       <c r="G32">
-        <v>7.066129787775949</v>
+        <v>7.497995853424072</v>
       </c>
       <c r="H32">
-        <v>11.89873609028827</v>
+        <v>12.58888339996338</v>
       </c>
       <c r="I32">
-        <v>12.26113936608195</v>
+        <v>9.676630973815918</v>
       </c>
       <c r="J32">
-        <v>12.98171593248749</v>
+        <v>11.34859085083008</v>
       </c>
       <c r="K32">
-        <v>14.90455612008368</v>
+        <v>13.13982582092285</v>
       </c>
       <c r="L32" t="s">
         <v>225</v>
@@ -82224,37 +82224,37 @@
     </row>
     <row r="33" spans="1:12">
       <c r="A33">
-        <v>11.2094301259305</v>
+        <v>9.025842666625977</v>
       </c>
       <c r="B33">
-        <v>11.26817515990196</v>
+        <v>9.202888488769531</v>
       </c>
       <c r="C33">
-        <v>8.771473592403817</v>
+        <v>8.69761848449707</v>
       </c>
       <c r="D33">
-        <v>5.853747262993734</v>
+        <v>6.301746845245361</v>
       </c>
       <c r="E33">
-        <v>6.820137645528917</v>
+        <v>7.653064250946045</v>
       </c>
       <c r="F33">
-        <v>7.817935876061367</v>
+        <v>7.967038631439209</v>
       </c>
       <c r="G33">
-        <v>6.967653467074832</v>
+        <v>7.496004581451416</v>
       </c>
       <c r="H33">
-        <v>11.86728868352966</v>
+        <v>12.57269477844238</v>
       </c>
       <c r="I33">
-        <v>12.16258506503183</v>
+        <v>9.650081634521484</v>
       </c>
       <c r="J33">
-        <v>12.98457659371835</v>
+        <v>11.30533409118652</v>
       </c>
       <c r="K33">
-        <v>14.91895301456682</v>
+        <v>13.0855770111084</v>
       </c>
       <c r="L33" t="s">
         <v>225</v>
@@ -82262,37 +82262,37 @@
     </row>
     <row r="34" spans="1:12">
       <c r="A34">
-        <v>11.0746099732053</v>
+        <v>9.018891334533691</v>
       </c>
       <c r="B34">
-        <v>11.18582473230827</v>
+        <v>9.171717643737793</v>
       </c>
       <c r="C34">
-        <v>8.67740167989956</v>
+        <v>8.697709083557129</v>
       </c>
       <c r="D34">
-        <v>5.805628030600949</v>
+        <v>6.302690029144287</v>
       </c>
       <c r="E34">
-        <v>6.767215268990861</v>
+        <v>7.62553071975708</v>
       </c>
       <c r="F34">
-        <v>7.778227904567685</v>
+        <v>7.951223850250244</v>
       </c>
       <c r="G34">
-        <v>6.976912699893052</v>
+        <v>7.495985507965088</v>
       </c>
       <c r="H34">
-        <v>11.81731756070607</v>
+        <v>12.55204105377197</v>
       </c>
       <c r="I34">
-        <v>12.08528509834597</v>
+        <v>9.644167900085449</v>
       </c>
       <c r="J34">
-        <v>13.05069550271297</v>
+        <v>11.28937530517578</v>
       </c>
       <c r="K34">
-        <v>15.0102855247749</v>
+        <v>13.06475448608398</v>
       </c>
       <c r="L34" t="s">
         <v>225</v>
@@ -82300,37 +82300,37 @@
     </row>
     <row r="35" spans="1:12">
       <c r="A35">
-        <v>11.10095590872969</v>
+        <v>9.024898529052734</v>
       </c>
       <c r="B35">
-        <v>11.25804755072256</v>
+        <v>9.154593467712402</v>
       </c>
       <c r="C35">
-        <v>8.677780256064185</v>
+        <v>8.699029922485352</v>
       </c>
       <c r="D35">
-        <v>5.758772594024708</v>
+        <v>6.299555778503418</v>
       </c>
       <c r="E35">
-        <v>6.704550497657054</v>
+        <v>7.612209796905518</v>
       </c>
       <c r="F35">
-        <v>7.657350732402714</v>
+        <v>7.951574325561523</v>
       </c>
       <c r="G35">
-        <v>6.802394763324311</v>
+        <v>7.490697383880615</v>
       </c>
       <c r="H35">
-        <v>11.76656847616301</v>
+        <v>12.54813575744629</v>
       </c>
       <c r="I35">
-        <v>11.99644840757845</v>
+        <v>9.645237922668457</v>
       </c>
       <c r="J35">
-        <v>13.03655854570065</v>
+        <v>11.28520202636719</v>
       </c>
       <c r="K35">
-        <v>14.95002716920066</v>
+        <v>13.05291938781738</v>
       </c>
       <c r="L35" t="s">
         <v>225</v>
@@ -82338,37 +82338,37 @@
     </row>
     <row r="36" spans="1:12">
       <c r="A36">
-        <v>10.93787732346567</v>
+        <v>9.016650199890137</v>
       </c>
       <c r="B36">
-        <v>11.19640181754126</v>
+        <v>9.14687442779541</v>
       </c>
       <c r="C36">
-        <v>8.591248775054847</v>
+        <v>8.700512886047363</v>
       </c>
       <c r="D36">
-        <v>5.684096819465887</v>
+        <v>6.306241512298584</v>
       </c>
       <c r="E36">
-        <v>6.586171654854675</v>
+        <v>7.618286609649658</v>
       </c>
       <c r="F36">
-        <v>7.60047754574959</v>
+        <v>7.945222854614258</v>
       </c>
       <c r="G36">
-        <v>6.899075720355814</v>
+        <v>7.499965667724609</v>
       </c>
       <c r="H36">
-        <v>11.69990329406669</v>
+        <v>12.53052997589111</v>
       </c>
       <c r="I36">
-        <v>12.04152551945507</v>
+        <v>9.640500068664551</v>
       </c>
       <c r="J36">
-        <v>12.98549435709208</v>
+        <v>11.27965354919434</v>
       </c>
       <c r="K36">
-        <v>14.93650493282426</v>
+        <v>13.05530738830566</v>
       </c>
       <c r="L36" t="s">
         <v>225</v>
@@ -82376,37 +82376,37 @@
     </row>
     <row r="37" spans="1:12">
       <c r="A37">
-        <v>11.0723684452649</v>
+        <v>9.032404899597168</v>
       </c>
       <c r="B37">
-        <v>11.07615886692201</v>
+        <v>9.171368598937988</v>
       </c>
       <c r="C37">
-        <v>8.56363139188618</v>
+        <v>8.712209701538086</v>
       </c>
       <c r="D37">
-        <v>5.64145082652358</v>
+        <v>6.305806636810303</v>
       </c>
       <c r="E37">
-        <v>6.576933737071594</v>
+        <v>7.647451400756836</v>
       </c>
       <c r="F37">
-        <v>7.428220573819801</v>
+        <v>7.972999572753906</v>
       </c>
       <c r="G37">
-        <v>6.79689274134274</v>
+        <v>7.508429050445557</v>
       </c>
       <c r="H37">
-        <v>11.64336924870751</v>
+        <v>12.55533885955811</v>
       </c>
       <c r="I37">
-        <v>11.97252796451826</v>
+        <v>9.657042503356934</v>
       </c>
       <c r="J37">
-        <v>12.9623458908056</v>
+        <v>11.29338073730469</v>
       </c>
       <c r="K37">
-        <v>14.84164494124893</v>
+        <v>13.07588195800781</v>
       </c>
       <c r="L37" t="s">
         <v>225</v>
@@ -82414,37 +82414,37 @@
     </row>
     <row r="38" spans="1:12">
       <c r="A38">
-        <v>10.93886416876838</v>
+        <v>9.020401954650879</v>
       </c>
       <c r="B38">
-        <v>11.04772804338261</v>
+        <v>9.138636589050293</v>
       </c>
       <c r="C38">
-        <v>8.547377467910884</v>
+        <v>8.701047897338867</v>
       </c>
       <c r="D38">
-        <v>5.566065291213092</v>
+        <v>6.307087421417236</v>
       </c>
       <c r="E38">
-        <v>6.578479316953527</v>
+        <v>7.617092609405518</v>
       </c>
       <c r="F38">
-        <v>7.509854422126175</v>
+        <v>7.947929382324219</v>
       </c>
       <c r="G38">
-        <v>6.775986015435521</v>
+        <v>7.501560688018799</v>
       </c>
       <c r="H38">
-        <v>11.58663585809988</v>
+        <v>12.53714942932129</v>
       </c>
       <c r="I38">
-        <v>11.8857908564063</v>
+        <v>9.650187492370605</v>
       </c>
       <c r="J38">
-        <v>12.96117167028656</v>
+        <v>11.28095245361328</v>
       </c>
       <c r="K38">
-        <v>14.84839962401306</v>
+        <v>13.05657958984375</v>
       </c>
       <c r="L38" t="s">
         <v>225</v>
@@ -82452,37 +82452,37 @@
     </row>
     <row r="39" spans="1:12">
       <c r="A39">
-        <v>10.91632003279532</v>
+        <v>9.005806922912598</v>
       </c>
       <c r="B39">
-        <v>11.02282797146295</v>
+        <v>9.120968818664551</v>
       </c>
       <c r="C39">
-        <v>8.511376306094673</v>
+        <v>8.682915687561035</v>
       </c>
       <c r="D39">
-        <v>5.583804136348466</v>
+        <v>6.303017616271973</v>
       </c>
       <c r="E39">
-        <v>6.619332198718535</v>
+        <v>7.595252513885498</v>
       </c>
       <c r="F39">
-        <v>7.477108745159268</v>
+        <v>7.94100284576416</v>
       </c>
       <c r="G39">
-        <v>7.081812315552754</v>
+        <v>7.509932041168213</v>
       </c>
       <c r="H39">
-        <v>11.55965053544358</v>
+        <v>12.52997589111328</v>
       </c>
       <c r="I39">
-        <v>11.8562787371571</v>
+        <v>9.641665458679199</v>
       </c>
       <c r="J39">
-        <v>13.00662325283336</v>
+        <v>11.26937103271484</v>
       </c>
       <c r="K39">
-        <v>14.91492363691424</v>
+        <v>13.05599403381348</v>
       </c>
       <c r="L39" t="s">
         <v>225</v>
@@ -82490,37 +82490,37 @@
     </row>
     <row r="40" spans="1:12">
       <c r="A40">
-        <v>10.8882880845704</v>
+        <v>9.010329246520996</v>
       </c>
       <c r="B40">
-        <v>10.97547062669363</v>
+        <v>9.141850471496582</v>
       </c>
       <c r="C40">
-        <v>8.412301699083107</v>
+        <v>8.688112258911133</v>
       </c>
       <c r="D40">
-        <v>5.559331124350086</v>
+        <v>6.304576396942139</v>
       </c>
       <c r="E40">
-        <v>6.466663019137557</v>
+        <v>7.618762969970703</v>
       </c>
       <c r="F40">
-        <v>7.421595964642156</v>
+        <v>7.950278282165527</v>
       </c>
       <c r="G40">
-        <v>7.019760370471214</v>
+        <v>7.510376453399658</v>
       </c>
       <c r="H40">
-        <v>11.52416264618905</v>
+        <v>12.53052234649658</v>
       </c>
       <c r="I40">
-        <v>11.82489356248883</v>
+        <v>9.64188289642334</v>
       </c>
       <c r="J40">
-        <v>12.88107848504346</v>
+        <v>11.27691841125488</v>
       </c>
       <c r="K40">
-        <v>14.72507337488973</v>
+        <v>13.06304168701172</v>
       </c>
       <c r="L40" t="s">
         <v>225</v>
@@ -82528,37 +82528,37 @@
     </row>
     <row r="41" spans="1:12">
       <c r="A41">
-        <v>10.97051360711099</v>
+        <v>9.010602951049805</v>
       </c>
       <c r="B41">
-        <v>11.13832898537255</v>
+        <v>9.122429847717285</v>
       </c>
       <c r="C41">
-        <v>8.542189289657497</v>
+        <v>8.691919326782227</v>
       </c>
       <c r="D41">
-        <v>5.647655541041471</v>
+        <v>6.309928417205811</v>
       </c>
       <c r="E41">
-        <v>6.621553576907891</v>
+        <v>7.592512607574463</v>
       </c>
       <c r="F41">
-        <v>7.549505970975707</v>
+        <v>7.945582389831543</v>
       </c>
       <c r="G41">
-        <v>6.849288833571178</v>
+        <v>7.490259170532227</v>
       </c>
       <c r="H41">
-        <v>11.49006105519821</v>
+        <v>12.52807235717773</v>
       </c>
       <c r="I41">
-        <v>11.8389464484405</v>
+        <v>9.643996238708496</v>
       </c>
       <c r="J41">
-        <v>13.00664820125201</v>
+        <v>11.27058219909668</v>
       </c>
       <c r="K41">
-        <v>14.92125770323351</v>
+        <v>13.03747940063477</v>
       </c>
       <c r="L41" t="s">
         <v>225</v>
@@ -82566,37 +82566,37 @@
     </row>
     <row r="42" spans="1:12">
       <c r="A42">
-        <v>10.08418742010263</v>
+        <v>8.010161399841309</v>
       </c>
       <c r="B42">
-        <v>9.528874899830573</v>
+        <v>7.198283672332764</v>
       </c>
       <c r="C42">
-        <v>6.316362198774944</v>
+        <v>8.181350708007812</v>
       </c>
       <c r="D42">
-        <v>4.944145677827415</v>
+        <v>7.571544647216797</v>
       </c>
       <c r="E42">
-        <v>4.834516858105339</v>
+        <v>7.40792989730835</v>
       </c>
       <c r="F42">
-        <v>4.907451057861025</v>
+        <v>5.404920101165771</v>
       </c>
       <c r="G42">
-        <v>6.275900523352274</v>
+        <v>6.72114896774292</v>
       </c>
       <c r="H42">
-        <v>11.22873801985581</v>
+        <v>12.65377426147461</v>
       </c>
       <c r="I42">
-        <v>10.40244300373163</v>
+        <v>10.08290481567383</v>
       </c>
       <c r="J42">
-        <v>11.55803690903381</v>
+        <v>9.732550621032715</v>
       </c>
       <c r="K42">
-        <v>12.26338197548171</v>
+        <v>10.98728179931641</v>
       </c>
       <c r="L42" t="s">
         <v>226</v>
@@ -82604,37 +82604,37 @@
     </row>
     <row r="43" spans="1:12">
       <c r="A43">
-        <v>10.14009560918863</v>
+        <v>8.055371284484863</v>
       </c>
       <c r="B43">
-        <v>9.54570084796336</v>
+        <v>7.274336338043213</v>
       </c>
       <c r="C43">
-        <v>6.42648845745769</v>
+        <v>8.094818115234375</v>
       </c>
       <c r="D43">
-        <v>4.901586112321655</v>
+        <v>7.513265609741211</v>
       </c>
       <c r="E43">
-        <v>4.482374671322232</v>
+        <v>7.292334079742432</v>
       </c>
       <c r="F43">
-        <v>5.135413934072721</v>
+        <v>5.304311752319336</v>
       </c>
       <c r="G43">
-        <v>6.252403223257573</v>
+        <v>6.724452495574951</v>
       </c>
       <c r="H43">
-        <v>11.19792243974955</v>
+        <v>12.59295654296875</v>
       </c>
       <c r="I43">
-        <v>10.39329380907804</v>
+        <v>10.04583644866943</v>
       </c>
       <c r="J43">
-        <v>11.43955397846744</v>
+        <v>9.744722366333008</v>
       </c>
       <c r="K43">
-        <v>12.23970619779722</v>
+        <v>10.93980598449707</v>
       </c>
       <c r="L43" t="s">
         <v>226</v>
@@ -82642,37 +82642,37 @@
     </row>
     <row r="44" spans="1:12">
       <c r="A44">
-        <v>9.950424142755416</v>
+        <v>8.012508392333984</v>
       </c>
       <c r="B44">
-        <v>9.245063775838817</v>
+        <v>7.177807331085205</v>
       </c>
       <c r="C44">
-        <v>6.264878690027484</v>
+        <v>8.088850975036621</v>
       </c>
       <c r="D44">
-        <v>5.065625413464763</v>
+        <v>7.523220539093018</v>
       </c>
       <c r="E44">
-        <v>4.633649765301315</v>
+        <v>7.326098918914795</v>
       </c>
       <c r="F44">
-        <v>4.847731977005544</v>
+        <v>5.298162460327148</v>
       </c>
       <c r="G44">
-        <v>6.047284704771343</v>
+        <v>6.715312004089355</v>
       </c>
       <c r="H44">
-        <v>11.18194611478861</v>
+        <v>12.60639095306396</v>
       </c>
       <c r="I44">
-        <v>10.30954508512625</v>
+        <v>10.04103851318359</v>
       </c>
       <c r="J44">
-        <v>11.38411939326813</v>
+        <v>9.691975593566895</v>
       </c>
       <c r="K44">
-        <v>12.23836234169777</v>
+        <v>10.91168785095215</v>
       </c>
       <c r="L44" t="s">
         <v>226</v>
@@ -82680,37 +82680,37 @@
     </row>
     <row r="45" spans="1:12">
       <c r="A45">
-        <v>9.955710959235084</v>
+        <v>8.042323112487793</v>
       </c>
       <c r="B45">
-        <v>9.170212615583528</v>
+        <v>7.292638778686523</v>
       </c>
       <c r="C45">
-        <v>6.324358962381311</v>
+        <v>7.888564109802246</v>
       </c>
       <c r="D45">
-        <v>4.972894804170076</v>
+        <v>7.42690896987915</v>
       </c>
       <c r="E45">
-        <v>4.922411182040633</v>
+        <v>7.091639041900635</v>
       </c>
       <c r="F45">
-        <v>5.051195983891169</v>
+        <v>5.439604759216309</v>
       </c>
       <c r="G45">
-        <v>6.792192027780253</v>
+        <v>6.816500186920166</v>
       </c>
       <c r="H45">
-        <v>11.16832495011834</v>
+        <v>12.49071598052979</v>
       </c>
       <c r="I45">
-        <v>10.39022538077303</v>
+        <v>9.855843544006348</v>
       </c>
       <c r="J45">
-        <v>11.42218593979168</v>
+        <v>9.675886154174805</v>
       </c>
       <c r="K45">
-        <v>12.16239356300158</v>
+        <v>10.79148483276367</v>
       </c>
       <c r="L45" t="s">
         <v>226</v>
@@ -82718,37 +82718,37 @@
     </row>
     <row r="46" spans="1:12">
       <c r="A46">
-        <v>9.803360208805678</v>
+        <v>7.943947315216064</v>
       </c>
       <c r="B46">
-        <v>9.165807751590989</v>
+        <v>7.082338809967041</v>
       </c>
       <c r="C46">
-        <v>6.395447056709929</v>
+        <v>7.916723251342773</v>
       </c>
       <c r="D46">
-        <v>5.265625065285453</v>
+        <v>7.285974979400635</v>
       </c>
       <c r="E46">
-        <v>4.806749695626233</v>
+        <v>7.255650997161865</v>
       </c>
       <c r="F46">
-        <v>4.618157252482636</v>
+        <v>5.26398229598999</v>
       </c>
       <c r="G46">
-        <v>5.94276700364912</v>
+        <v>6.753415107727051</v>
       </c>
       <c r="H46">
-        <v>11.15751638591493</v>
+        <v>12.55828762054443</v>
       </c>
       <c r="I46">
-        <v>10.34909887487647</v>
+        <v>9.86160945892334</v>
       </c>
       <c r="J46">
-        <v>11.39255157720316</v>
+        <v>9.593631744384766</v>
       </c>
       <c r="K46">
-        <v>12.23329322596923</v>
+        <v>10.81208992004395</v>
       </c>
       <c r="L46" t="s">
         <v>226</v>
@@ -82756,37 +82756,37 @@
     </row>
     <row r="47" spans="1:12">
       <c r="A47">
-        <v>9.959395184474424</v>
+        <v>8.069658279418945</v>
       </c>
       <c r="B47">
-        <v>9.426168349614136</v>
+        <v>7.431924819946289</v>
       </c>
       <c r="C47">
-        <v>6.338201421618375</v>
+        <v>7.675036907196045</v>
       </c>
       <c r="D47">
-        <v>5.039455618995378</v>
+        <v>7.02784538269043</v>
       </c>
       <c r="E47">
-        <v>4.607389720996889</v>
+        <v>6.82960319519043</v>
       </c>
       <c r="F47">
-        <v>5.04700277019989</v>
+        <v>5.105464935302734</v>
       </c>
       <c r="G47">
-        <v>6.848765070783797</v>
+        <v>6.885118961334229</v>
       </c>
       <c r="H47">
-        <v>11.14203568150175</v>
+        <v>12.37507724761963</v>
       </c>
       <c r="I47">
-        <v>10.42972709907212</v>
+        <v>9.639530181884766</v>
       </c>
       <c r="J47">
-        <v>11.41950571817091</v>
+        <v>9.574289321899414</v>
       </c>
       <c r="K47">
-        <v>12.16024392470548</v>
+        <v>10.69454002380371</v>
       </c>
       <c r="L47" t="s">
         <v>226</v>
@@ -82794,37 +82794,37 @@
     </row>
     <row r="48" spans="1:12">
       <c r="A48">
-        <v>9.945109227226947</v>
+        <v>8.00373649597168</v>
       </c>
       <c r="B48">
-        <v>8.836050913646645</v>
+        <v>7.370974540710449</v>
       </c>
       <c r="C48">
-        <v>6.260643232884843</v>
+        <v>7.58307933807373</v>
       </c>
       <c r="D48">
-        <v>5.047003088643059</v>
+        <v>6.817726612091064</v>
       </c>
       <c r="E48">
-        <v>4.383414421252465</v>
+        <v>6.809332370758057</v>
       </c>
       <c r="F48">
-        <v>4.310930976148011</v>
+        <v>5.193692207336426</v>
       </c>
       <c r="G48">
-        <v>6.908495782519482</v>
+        <v>6.905392169952393</v>
       </c>
       <c r="H48">
-        <v>11.12630337387954</v>
+        <v>12.29521465301514</v>
       </c>
       <c r="I48">
-        <v>10.14145401960482</v>
+        <v>9.511515617370605</v>
       </c>
       <c r="J48">
-        <v>11.39892277977632</v>
+        <v>9.501901626586914</v>
       </c>
       <c r="K48">
-        <v>12.25511145497528</v>
+        <v>10.59213256835938</v>
       </c>
       <c r="L48" t="s">
         <v>226</v>
@@ -82832,37 +82832,37 @@
     </row>
     <row r="49" spans="1:12">
       <c r="A49">
-        <v>9.749105370914396</v>
+        <v>7.999686717987061</v>
       </c>
       <c r="B49">
-        <v>8.865342979257637</v>
+        <v>7.346251964569092</v>
       </c>
       <c r="C49">
-        <v>6.228291847428324</v>
+        <v>7.569989681243896</v>
       </c>
       <c r="D49">
-        <v>5.126467109621378</v>
+        <v>6.832676410675049</v>
       </c>
       <c r="E49">
-        <v>4.525405398024628</v>
+        <v>6.829832077026367</v>
       </c>
       <c r="F49">
-        <v>4.494713044438368</v>
+        <v>5.230521202087402</v>
       </c>
       <c r="G49">
-        <v>6.746832721662815</v>
+        <v>6.90844202041626</v>
       </c>
       <c r="H49">
-        <v>11.11110869382991</v>
+        <v>12.30592441558838</v>
       </c>
       <c r="I49">
-        <v>10.23263143078527</v>
+        <v>9.509160041809082</v>
       </c>
       <c r="J49">
-        <v>11.40957527170402</v>
+        <v>9.492105484008789</v>
       </c>
       <c r="K49">
-        <v>12.24533075221508</v>
+        <v>10.58953666687012</v>
       </c>
       <c r="L49" t="s">
         <v>226</v>
@@ -82870,37 +82870,37 @@
     </row>
     <row r="50" spans="1:12">
       <c r="A50">
-        <v>9.68415616319025</v>
+        <v>8.692324638366699</v>
       </c>
       <c r="B50">
-        <v>8.895020674639253</v>
+        <v>8.188955307006836</v>
       </c>
       <c r="C50">
-        <v>6.281643562102488</v>
+        <v>7.464807987213135</v>
       </c>
       <c r="D50">
-        <v>4.914545125969586</v>
+        <v>6.561419010162354</v>
       </c>
       <c r="E50">
-        <v>4.384800284548258</v>
+        <v>7.00120735168457</v>
       </c>
       <c r="F50">
-        <v>2.975928646257311</v>
+        <v>5.424391269683838</v>
       </c>
       <c r="G50">
-        <v>6.751173721037365</v>
+        <v>7.728869915008545</v>
       </c>
       <c r="H50">
-        <v>11.09845829259199</v>
+        <v>12.81477642059326</v>
       </c>
       <c r="I50">
-        <v>10.06219924369095</v>
+        <v>9.291567802429199</v>
       </c>
       <c r="J50">
-        <v>11.35005353199759</v>
+        <v>10.26482582092285</v>
       </c>
       <c r="K50">
-        <v>12.2250961017043</v>
+        <v>11.76234817504883</v>
       </c>
       <c r="L50" t="s">
         <v>226</v>
@@ -82908,37 +82908,37 @@
     </row>
     <row r="51" spans="1:12">
       <c r="A51">
-        <v>9.837763155191903</v>
+        <v>7.951871871948242</v>
       </c>
       <c r="B51">
-        <v>9.112114786503703</v>
+        <v>7.121503353118896</v>
       </c>
       <c r="C51">
-        <v>6.324358962381311</v>
+        <v>7.892995357513428</v>
       </c>
       <c r="D51">
-        <v>5.112481008491698</v>
+        <v>7.273538112640381</v>
       </c>
       <c r="E51">
-        <v>4.687262023529489</v>
+        <v>7.180722236633301</v>
       </c>
       <c r="F51">
-        <v>4.544545564171656</v>
+        <v>5.278271198272705</v>
       </c>
       <c r="G51">
-        <v>6.104021357215002</v>
+        <v>6.751991748809814</v>
       </c>
       <c r="H51">
-        <v>11.08971720704553</v>
+        <v>12.49582290649414</v>
       </c>
       <c r="I51">
-        <v>10.21773039392608</v>
+        <v>9.818228721618652</v>
       </c>
       <c r="J51">
-        <v>11.26578801097352</v>
+        <v>9.575199127197266</v>
       </c>
       <c r="K51">
-        <v>12.14901422786691</v>
+        <v>10.76286697387695</v>
       </c>
       <c r="L51" t="s">
         <v>226</v>
@@ -82946,37 +82946,37 @@
     </row>
     <row r="52" spans="1:12">
       <c r="A52">
-        <v>9.649956376226669</v>
+        <v>7.872829914093018</v>
       </c>
       <c r="B52">
-        <v>8.328182673317123</v>
+        <v>6.278491497039795</v>
       </c>
       <c r="C52">
-        <v>6.147280411174668</v>
+        <v>7.459364414215088</v>
       </c>
       <c r="D52">
-        <v>5.129933282995787</v>
+        <v>6.782326221466064</v>
       </c>
       <c r="E52">
-        <v>5.63677174457126</v>
+        <v>7.614556789398193</v>
       </c>
       <c r="F52">
-        <v>4.302120437290235</v>
+        <v>5.163017272949219</v>
       </c>
       <c r="G52">
-        <v>5.362855887685608</v>
+        <v>7.151439189910889</v>
       </c>
       <c r="H52">
-        <v>11.08296272551786</v>
+        <v>12.72250461578369</v>
       </c>
       <c r="I52">
-        <v>10.91891949824172</v>
+        <v>9.88410472869873</v>
       </c>
       <c r="J52">
-        <v>11.28271534164552</v>
+        <v>9.796917915344238</v>
       </c>
       <c r="K52">
-        <v>12.07078733282954</v>
+        <v>11.00533294677734</v>
       </c>
       <c r="L52" t="s">
         <v>227</v>
@@ -82984,37 +82984,37 @@
     </row>
     <row r="53" spans="1:12">
       <c r="A53">
-        <v>9.502097480179991</v>
+        <v>7.815477848052979</v>
       </c>
       <c r="B53">
-        <v>7.676834267495703</v>
+        <v>6.388833999633789</v>
       </c>
       <c r="C53">
-        <v>5.933423273073401</v>
+        <v>7.581580638885498</v>
       </c>
       <c r="D53">
-        <v>4.861669511998643</v>
+        <v>7.010202884674072</v>
       </c>
       <c r="E53">
-        <v>5.51923624511185</v>
+        <v>7.460376739501953</v>
       </c>
       <c r="F53">
-        <v>4.293230778747829</v>
+        <v>5.104201316833496</v>
       </c>
       <c r="G53">
-        <v>5.220021835376039</v>
+        <v>6.930280208587646</v>
       </c>
       <c r="H53">
-        <v>11.01144492870357</v>
+        <v>12.66789531707764</v>
       </c>
       <c r="I53">
-        <v>10.44419553784319</v>
+        <v>9.872798919677734</v>
       </c>
       <c r="J53">
-        <v>11.25290178818903</v>
+        <v>9.678245544433594</v>
       </c>
       <c r="K53">
-        <v>11.98302631448992</v>
+        <v>10.88164138793945</v>
       </c>
       <c r="L53" t="s">
         <v>227</v>
@@ -83022,37 +83022,37 @@
     </row>
     <row r="54" spans="1:12">
       <c r="A54">
-        <v>9.626049101257038</v>
+        <v>7.788483142852783</v>
       </c>
       <c r="B54">
-        <v>8.525822452020437</v>
+        <v>6.308689594268799</v>
       </c>
       <c r="C54">
-        <v>5.784508641026316</v>
+        <v>7.443159103393555</v>
       </c>
       <c r="D54">
-        <v>4.897228458367167</v>
+        <v>6.738519191741943</v>
       </c>
       <c r="E54">
-        <v>5.475998590297116</v>
+        <v>7.426239490509033</v>
       </c>
       <c r="F54">
-        <v>4.319664566871934</v>
+        <v>5.118626117706299</v>
       </c>
       <c r="G54">
-        <v>5.213323952101721</v>
+        <v>6.927225112915039</v>
       </c>
       <c r="H54">
-        <v>10.96622316007153</v>
+        <v>12.59139537811279</v>
       </c>
       <c r="I54">
-        <v>10.28799381718775</v>
+        <v>9.931796073913574</v>
       </c>
       <c r="J54">
-        <v>11.22632428814024</v>
+        <v>9.638177871704102</v>
       </c>
       <c r="K54">
-        <v>12.02197618051813</v>
+        <v>10.82966232299805</v>
       </c>
       <c r="L54" t="s">
         <v>227</v>
@@ -83060,37 +83060,37 @@
     </row>
     <row r="55" spans="1:12">
       <c r="A55">
-        <v>9.492088171408042</v>
+        <v>7.803560733795166</v>
       </c>
       <c r="B55">
-        <v>7.74788479377561</v>
+        <v>6.326603412628174</v>
       </c>
       <c r="C55">
-        <v>5.497623449531776</v>
+        <v>7.43656063079834</v>
       </c>
       <c r="D55">
-        <v>4.678442169703089</v>
+        <v>6.739330768585205</v>
       </c>
       <c r="E55">
-        <v>5.148785503544806</v>
+        <v>7.303601741790771</v>
       </c>
       <c r="F55">
-        <v>4.219123548352339</v>
+        <v>4.998278617858887</v>
       </c>
       <c r="G55">
-        <v>5.053332152183128</v>
+        <v>6.795888423919678</v>
       </c>
       <c r="H55">
-        <v>10.90837913784601</v>
+        <v>12.5523681640625</v>
       </c>
       <c r="I55">
-        <v>9.823722602117806</v>
+        <v>9.777718544006348</v>
       </c>
       <c r="J55">
-        <v>11.22898453238628</v>
+        <v>9.566774368286133</v>
       </c>
       <c r="K55">
-        <v>11.96126556914806</v>
+        <v>10.78903198242188</v>
       </c>
       <c r="L55" t="s">
         <v>227</v>
@@ -83098,37 +83098,37 @@
     </row>
     <row r="56" spans="1:12">
       <c r="A56">
-        <v>9.490410194631801</v>
+        <v>7.78729772567749</v>
       </c>
       <c r="B56">
-        <v>7.544919766036737</v>
+        <v>6.196729183197021</v>
       </c>
       <c r="C56">
-        <v>5.178657320409132</v>
+        <v>7.337668895721436</v>
       </c>
       <c r="D56">
-        <v>4.639656531550772</v>
+        <v>6.663179397583008</v>
       </c>
       <c r="E56">
-        <v>5.15200637589447</v>
+        <v>7.298375606536865</v>
       </c>
       <c r="F56">
-        <v>3.878797087529519</v>
+        <v>4.931769371032715</v>
       </c>
       <c r="G56">
-        <v>4.685782987537485</v>
+        <v>6.816959857940674</v>
       </c>
       <c r="H56">
-        <v>10.86012016401381</v>
+        <v>12.55109405517578</v>
       </c>
       <c r="I56">
-        <v>9.604632157014311</v>
+        <v>9.709835052490234</v>
       </c>
       <c r="J56">
-        <v>11.12927077601804</v>
+        <v>9.570186614990234</v>
       </c>
       <c r="K56">
-        <v>11.91023891843687</v>
+        <v>10.77782440185547</v>
       </c>
       <c r="L56" t="s">
         <v>227</v>
@@ -83136,37 +83136,37 @@
     </row>
     <row r="57" spans="1:12">
       <c r="A57">
-        <v>9.233297039661309</v>
+        <v>7.779971599578857</v>
       </c>
       <c r="B57">
-        <v>8.120026853064916</v>
+        <v>6.209316730499268</v>
       </c>
       <c r="C57">
-        <v>4.793952493777613</v>
+        <v>7.219605922698975</v>
       </c>
       <c r="D57">
-        <v>4.383487409328144</v>
+        <v>6.527446746826172</v>
       </c>
       <c r="E57">
-        <v>5.214331770897902</v>
+        <v>7.325973987579346</v>
       </c>
       <c r="F57">
-        <v>3.717866990987189</v>
+        <v>5.045633316040039</v>
       </c>
       <c r="G57">
-        <v>4.872271928811614</v>
+        <v>6.789758205413818</v>
       </c>
       <c r="H57">
-        <v>10.8247326582071</v>
+        <v>12.55798053741455</v>
       </c>
       <c r="I57">
-        <v>8.374092270852485</v>
+        <v>9.575045585632324</v>
       </c>
       <c r="J57">
-        <v>11.1278020594193</v>
+        <v>9.637493133544922</v>
       </c>
       <c r="K57">
-        <v>11.9213786975178</v>
+        <v>10.74742126464844</v>
       </c>
       <c r="L57" t="s">
         <v>227</v>
@@ -83174,37 +83174,37 @@
     </row>
     <row r="58" spans="1:12">
       <c r="A58">
-        <v>9.329505208062027</v>
+        <v>7.719095706939697</v>
       </c>
       <c r="B58">
-        <v>7.594213639176506</v>
+        <v>6.246932029724121</v>
       </c>
       <c r="C58">
-        <v>4.724433902672853</v>
+        <v>7.332839965820312</v>
       </c>
       <c r="D58">
-        <v>4.506931617372412</v>
+        <v>6.731194496154785</v>
       </c>
       <c r="E58">
-        <v>5.208271207443793</v>
+        <v>7.368924140930176</v>
       </c>
       <c r="F58">
-        <v>3.905465078566059</v>
+        <v>5.010024547576904</v>
       </c>
       <c r="G58">
-        <v>4.564861948361049</v>
+        <v>6.797808170318604</v>
       </c>
       <c r="H58">
-        <v>10.79718042119968</v>
+        <v>12.50623989105225</v>
       </c>
       <c r="I58">
-        <v>8.83443411465325</v>
+        <v>9.860977172851562</v>
       </c>
       <c r="J58">
-        <v>11.12091937654622</v>
+        <v>9.572269439697266</v>
       </c>
       <c r="K58">
-        <v>11.85709813415508</v>
+        <v>10.73353576660156</v>
       </c>
       <c r="L58" t="s">
         <v>227</v>
@@ -83212,37 +83212,37 @@
     </row>
     <row r="59" spans="1:12">
       <c r="A59">
-        <v>9.374818510969016</v>
+        <v>7.743226528167725</v>
       </c>
       <c r="B59">
-        <v>7.74788479377561</v>
+        <v>6.264796733856201</v>
       </c>
       <c r="C59">
-        <v>4.890349128221754</v>
+        <v>7.313573360443115</v>
       </c>
       <c r="D59">
-        <v>4.519752180056637</v>
+        <v>6.69603967666626</v>
       </c>
       <c r="E59">
-        <v>4.995709794255508</v>
+        <v>7.352295875549316</v>
       </c>
       <c r="F59">
-        <v>3.95675902426953</v>
+        <v>5.005662441253662</v>
       </c>
       <c r="G59">
-        <v>4.486460471097104</v>
+        <v>6.796481132507324</v>
       </c>
       <c r="H59">
-        <v>10.76888257202916</v>
+        <v>12.51333808898926</v>
       </c>
       <c r="I59">
-        <v>8.804875313868017</v>
+        <v>9.810433387756348</v>
       </c>
       <c r="J59">
-        <v>11.11927363946135</v>
+        <v>9.577339172363281</v>
       </c>
       <c r="K59">
-        <v>11.89025017336155</v>
+        <v>10.73440742492676</v>
       </c>
       <c r="L59" t="s">
         <v>227</v>
@@ -83250,37 +83250,37 @@
     </row>
     <row r="60" spans="1:12">
       <c r="A60">
-        <v>9.315600882633676</v>
+        <v>7.800805568695068</v>
       </c>
       <c r="B60">
-        <v>8.687592121993916</v>
+        <v>6.18497371673584</v>
       </c>
       <c r="C60">
-        <v>4.803109974096709</v>
+        <v>7.0318922996521</v>
       </c>
       <c r="D60">
-        <v>4.361346504063206</v>
+        <v>6.508697032928467</v>
       </c>
       <c r="E60">
-        <v>4.995709794255508</v>
+        <v>7.303987979888916</v>
       </c>
       <c r="F60">
-        <v>4.159699845307038</v>
+        <v>4.857955455780029</v>
       </c>
       <c r="G60">
-        <v>4.614998397173735</v>
+        <v>6.653689861297607</v>
       </c>
       <c r="H60">
-        <v>10.73913446994158</v>
+        <v>12.48064231872559</v>
       </c>
       <c r="I60">
-        <v>8.374092270852485</v>
+        <v>9.514108657836914</v>
       </c>
       <c r="J60">
-        <v>11.05164809890053</v>
+        <v>9.535209655761719</v>
       </c>
       <c r="K60">
-        <v>11.78586607907556</v>
+        <v>10.65759468078613</v>
       </c>
       <c r="L60" t="s">
         <v>227</v>
@@ -83288,37 +83288,37 @@
     </row>
     <row r="61" spans="1:12">
       <c r="A61">
-        <v>9.350005700988769</v>
+        <v>7.738646030426025</v>
       </c>
       <c r="B61">
-        <v>8.061136332255126</v>
+        <v>6.231592655181885</v>
       </c>
       <c r="C61">
-        <v>4.890349128221754</v>
+        <v>7.302928447723389</v>
       </c>
       <c r="D61">
-        <v>4.426351329675406</v>
+        <v>6.70506763458252</v>
       </c>
       <c r="E61">
-        <v>5.132525144492178</v>
+        <v>7.3580641746521</v>
       </c>
       <c r="F61">
-        <v>3.969181419268095</v>
+        <v>5.012449264526367</v>
       </c>
       <c r="G61">
-        <v>4.762490124120882</v>
+        <v>6.801271915435791</v>
       </c>
       <c r="H61">
-        <v>10.72195717696396</v>
+        <v>12.51600074768066</v>
       </c>
       <c r="I61">
-        <v>9.103744538071304</v>
+        <v>9.816165924072266</v>
       </c>
       <c r="J61">
-        <v>11.08747871694408</v>
+        <v>9.585439682006836</v>
       </c>
       <c r="K61">
-        <v>11.7917685887548</v>
+        <v>10.73092079162598</v>
       </c>
       <c r="L61" t="s">
         <v>227</v>
@@ -83326,37 +83326,37 @@
     </row>
     <row r="62" spans="1:12">
       <c r="A62">
-        <v>9.475435979849951</v>
+        <v>7.7220778465271</v>
       </c>
       <c r="B62">
-        <v>8.536269280337514</v>
+        <v>6.877315521240234</v>
       </c>
       <c r="C62">
-        <v>5.489855486703791</v>
+        <v>7.352654457092285</v>
       </c>
       <c r="D62">
-        <v>4.653124411886033</v>
+        <v>7.136280059814453</v>
       </c>
       <c r="E62">
-        <v>5.205836605161545</v>
+        <v>7.243504047393799</v>
       </c>
       <c r="F62">
-        <v>3.851398383611711</v>
+        <v>5.284408092498779</v>
       </c>
       <c r="G62">
-        <v>5.022905630590479</v>
+        <v>6.712863922119141</v>
       </c>
       <c r="H62">
-        <v>10.59301708604476</v>
+        <v>12.59557628631592</v>
       </c>
       <c r="I62">
-        <v>10.66455295068265</v>
+        <v>9.596951484680176</v>
       </c>
       <c r="J62">
-        <v>11.05064305424883</v>
+        <v>9.321556091308594</v>
       </c>
       <c r="K62">
-        <v>11.50728738080219</v>
+        <v>10.45412635803223</v>
       </c>
       <c r="L62" t="s">
         <v>228</v>
@@ -83364,37 +83364,37 @@
     </row>
     <row r="63" spans="1:12">
       <c r="A63">
-        <v>9.525313288445897</v>
+        <v>7.723429203033447</v>
       </c>
       <c r="B63">
-        <v>8.086979959176965</v>
+        <v>6.581695079803467</v>
       </c>
       <c r="C63">
-        <v>5.471336624137617</v>
+        <v>7.077649116516113</v>
       </c>
       <c r="D63">
-        <v>4.449849435930655</v>
+        <v>6.597029209136963</v>
       </c>
       <c r="E63">
-        <v>5.106618580646732</v>
+        <v>7.097505569458008</v>
       </c>
       <c r="F63">
-        <v>3.878797087529519</v>
+        <v>4.985407829284668</v>
       </c>
       <c r="G63">
-        <v>5.523927207401756</v>
+        <v>6.739494800567627</v>
       </c>
       <c r="H63">
-        <v>10.51644849720619</v>
+        <v>12.63487243652344</v>
       </c>
       <c r="I63">
-        <v>10.05238636542146</v>
+        <v>9.415802001953125</v>
       </c>
       <c r="J63">
-        <v>10.75804472169611</v>
+        <v>9.427377700805664</v>
       </c>
       <c r="K63">
-        <v>11.41266304303183</v>
+        <v>10.57867813110352</v>
       </c>
       <c r="L63" t="s">
         <v>228</v>
@@ -83402,37 +83402,37 @@
     </row>
     <row r="64" spans="1:12">
       <c r="A64">
-        <v>9.629196880361024</v>
+        <v>7.766237735748291</v>
       </c>
       <c r="B64">
-        <v>8.43058573284058</v>
+        <v>6.867747783660889</v>
       </c>
       <c r="C64">
-        <v>5.485257823115336</v>
+        <v>7.345248699188232</v>
       </c>
       <c r="D64">
-        <v>4.449849435930655</v>
+        <v>6.9870924949646</v>
       </c>
       <c r="E64">
-        <v>4.988919878586549</v>
+        <v>7.283212661743164</v>
       </c>
       <c r="F64">
-        <v>3.892219978131886</v>
+        <v>5.248706340789795</v>
       </c>
       <c r="G64">
-        <v>4.754015388053651</v>
+        <v>6.682438373565674</v>
       </c>
       <c r="H64">
-        <v>10.47805450414053</v>
+        <v>12.57058048248291</v>
       </c>
       <c r="I64">
-        <v>10.26735877106746</v>
+        <v>9.584602355957031</v>
       </c>
       <c r="J64">
-        <v>10.82655526868931</v>
+        <v>9.329774856567383</v>
       </c>
       <c r="K64">
-        <v>11.38892313201553</v>
+        <v>10.53116798400879</v>
       </c>
       <c r="L64" t="s">
         <v>228</v>
@@ -83440,37 +83440,37 @@
     </row>
     <row r="65" spans="1:12">
       <c r="A65">
-        <v>9.475435979849951</v>
+        <v>7.746986865997314</v>
       </c>
       <c r="B65">
-        <v>8.766365437974503</v>
+        <v>6.652412891387939</v>
       </c>
       <c r="C65">
-        <v>5.494432108488017</v>
+        <v>6.599089622497559</v>
       </c>
       <c r="D65">
-        <v>4.442995469687976</v>
+        <v>5.943387031555176</v>
       </c>
       <c r="E65">
-        <v>4.969813299576001</v>
+        <v>6.636760234832764</v>
       </c>
       <c r="F65">
-        <v>3.701866810931057</v>
+        <v>4.391880035400391</v>
       </c>
       <c r="G65">
-        <v>5.518988530697036</v>
+        <v>6.597337245941162</v>
       </c>
       <c r="H65">
-        <v>10.45338964780307</v>
+        <v>12.37679481506348</v>
       </c>
       <c r="I65">
-        <v>9.985579436136893</v>
+        <v>8.826321601867676</v>
       </c>
       <c r="J65">
-        <v>10.74735095764213</v>
+        <v>9.164545059204102</v>
       </c>
       <c r="K65">
-        <v>11.33756628647258</v>
+        <v>10.46340179443359</v>
       </c>
       <c r="L65" t="s">
         <v>228</v>
@@ -83478,37 +83478,37 @@
     </row>
     <row r="66" spans="1:12">
       <c r="A66">
-        <v>9.286478018660565</v>
+        <v>7.691033363342285</v>
       </c>
       <c r="B66">
-        <v>8.766365437974503</v>
+        <v>6.77371072769165</v>
       </c>
       <c r="C66">
-        <v>5.489855486703791</v>
+        <v>7.18559741973877</v>
       </c>
       <c r="D66">
-        <v>4.619107866842239</v>
+        <v>6.51474666595459</v>
       </c>
       <c r="E66">
-        <v>5.109977636824892</v>
+        <v>6.811386585235596</v>
       </c>
       <c r="F66">
-        <v>4.465081543193338</v>
+        <v>5.059329032897949</v>
       </c>
       <c r="G66">
-        <v>5.94082074935416</v>
+        <v>6.604103565216064</v>
       </c>
       <c r="H66">
-        <v>10.41793992519053</v>
+        <v>12.32300853729248</v>
       </c>
       <c r="I66">
-        <v>9.902375834806907</v>
+        <v>9.200273513793945</v>
       </c>
       <c r="J66">
-        <v>10.66859356178021</v>
+        <v>9.077367782592773</v>
       </c>
       <c r="K66">
-        <v>11.23796216492622</v>
+        <v>10.23398017883301</v>
       </c>
       <c r="L66" t="s">
         <v>228</v>
@@ -83516,37 +83516,37 @@
     </row>
     <row r="67" spans="1:12">
       <c r="A67">
-        <v>9.258283606173082</v>
+        <v>7.746089458465576</v>
       </c>
       <c r="B67">
-        <v>8.589341559084353</v>
+        <v>6.832883358001709</v>
       </c>
       <c r="C67">
-        <v>5.594298283136826</v>
+        <v>7.309542179107666</v>
       </c>
       <c r="D67">
-        <v>4.577901217968692</v>
+        <v>6.470871925354004</v>
       </c>
       <c r="E67">
-        <v>4.633649765301315</v>
+        <v>6.869840145111084</v>
       </c>
       <c r="F67">
-        <v>4.005548706296048</v>
+        <v>5.252417087554932</v>
       </c>
       <c r="G67">
-        <v>5.620877805103573</v>
+        <v>6.649786472320557</v>
       </c>
       <c r="H67">
-        <v>10.37553769717745</v>
+        <v>12.28264617919922</v>
       </c>
       <c r="I67">
-        <v>9.732435614368235</v>
+        <v>9.119925498962402</v>
       </c>
       <c r="J67">
-        <v>10.66807645037777</v>
+        <v>9.131662368774414</v>
       </c>
       <c r="K67">
-        <v>11.24626531538726</v>
+        <v>10.19285202026367</v>
       </c>
       <c r="L67" t="s">
         <v>228</v>
@@ -83554,37 +83554,37 @@
     </row>
     <row r="68" spans="1:12">
       <c r="A68">
-        <v>9.338635868689765</v>
+        <v>7.719418048858643</v>
       </c>
       <c r="B68">
-        <v>8.806540576464949</v>
+        <v>6.807326793670654</v>
       </c>
       <c r="C68">
-        <v>5.530310445033498</v>
+        <v>7.038947582244873</v>
       </c>
       <c r="D68">
-        <v>4.318657254386125</v>
+        <v>6.399444103240967</v>
       </c>
       <c r="E68">
-        <v>4.755503876084042</v>
+        <v>6.714260578155518</v>
       </c>
       <c r="F68">
-        <v>4.310930976148011</v>
+        <v>4.865650653839111</v>
       </c>
       <c r="G68">
-        <v>6.388665228353801</v>
+        <v>6.628880023956299</v>
       </c>
       <c r="H68">
-        <v>10.3430498720107</v>
+        <v>12.27712249755859</v>
       </c>
       <c r="I68">
-        <v>9.876458897271496</v>
+        <v>9.120041847229004</v>
       </c>
       <c r="J68">
-        <v>10.5522183176278</v>
+        <v>9.07094669342041</v>
       </c>
       <c r="K68">
-        <v>11.20661164107952</v>
+        <v>10.23153114318848</v>
       </c>
       <c r="L68" t="s">
         <v>228</v>
@@ -83592,37 +83592,37 @@
     </row>
     <row r="69" spans="1:12">
       <c r="A69">
-        <v>9.193759262016293</v>
+        <v>7.765950202941895</v>
       </c>
       <c r="B69">
-        <v>8.536269280337514</v>
+        <v>6.989453792572021</v>
       </c>
       <c r="C69">
-        <v>5.685090190700641</v>
+        <v>7.080974578857422</v>
       </c>
       <c r="D69">
-        <v>4.229093196163867</v>
+        <v>6.253692150115967</v>
       </c>
       <c r="E69">
-        <v>4.769742655528466</v>
+        <v>6.63040828704834</v>
       </c>
       <c r="F69">
-        <v>4.558338749317682</v>
+        <v>4.73971700668335</v>
       </c>
       <c r="G69">
-        <v>6.371928416301866</v>
+        <v>6.845178127288818</v>
       </c>
       <c r="H69">
-        <v>10.32608287545382</v>
+        <v>12.25167751312256</v>
       </c>
       <c r="I69">
-        <v>9.669170686578848</v>
+        <v>9.101275444030762</v>
       </c>
       <c r="J69">
-        <v>10.54112202316581</v>
+        <v>9.125107765197754</v>
       </c>
       <c r="K69">
-        <v>11.11681644683265</v>
+        <v>10.34574699401855</v>
       </c>
       <c r="L69" t="s">
         <v>228</v>
@@ -83630,37 +83630,37 @@
     </row>
     <row r="70" spans="1:12">
       <c r="A70">
-        <v>9.119929331765611</v>
+        <v>7.755186557769775</v>
       </c>
       <c r="B70">
-        <v>8.97836165528059</v>
+        <v>6.893700122833252</v>
       </c>
       <c r="C70">
-        <v>5.718488476060484</v>
+        <v>7.300965309143066</v>
       </c>
       <c r="D70">
-        <v>4.422146488013859</v>
+        <v>6.604739189147949</v>
       </c>
       <c r="E70">
-        <v>4.77912349311153</v>
+        <v>6.779304981231689</v>
       </c>
       <c r="F70">
-        <v>4.362223757377671</v>
+        <v>5.087081909179688</v>
       </c>
       <c r="G70">
-        <v>6.194657286813926</v>
+        <v>6.681260108947754</v>
       </c>
       <c r="H70">
-        <v>10.30958209251049</v>
+        <v>12.31108283996582</v>
       </c>
       <c r="I70">
-        <v>9.612094870948034</v>
+        <v>9.287320137023926</v>
       </c>
       <c r="J70">
-        <v>10.53877018470768</v>
+        <v>9.163112640380859</v>
       </c>
       <c r="K70">
-        <v>11.12732833496401</v>
+        <v>10.32280731201172</v>
       </c>
       <c r="L70" t="s">
         <v>228</v>
@@ -83668,37 +83668,37 @@
     </row>
     <row r="71" spans="1:12">
       <c r="A71">
-        <v>9.188094763028863</v>
+        <v>7.653131484985352</v>
       </c>
       <c r="B71">
-        <v>8.879260908181543</v>
+        <v>6.719630241394043</v>
       </c>
       <c r="C71">
-        <v>5.673704981250983</v>
+        <v>6.748983860015869</v>
       </c>
       <c r="D71">
-        <v>4.203207621018538</v>
+        <v>5.896580219268799</v>
       </c>
       <c r="E71">
-        <v>5.136451753004676</v>
+        <v>6.571769237518311</v>
       </c>
       <c r="F71">
-        <v>4.530559463041977</v>
+        <v>4.46169900894165</v>
       </c>
       <c r="G71">
-        <v>6.421321048099339</v>
+        <v>6.630295753479004</v>
       </c>
       <c r="H71">
-        <v>10.29107152000966</v>
+        <v>12.21260643005371</v>
       </c>
       <c r="I71">
-        <v>10.07323032712322</v>
+        <v>8.83035945892334</v>
       </c>
       <c r="J71">
-        <v>10.57461632226369</v>
+        <v>8.948030471801758</v>
       </c>
       <c r="K71">
-        <v>11.1550434499571</v>
+        <v>10.27006721496582</v>
       </c>
       <c r="L71" t="s">
         <v>228</v>
@@ -83706,37 +83706,37 @@
     </row>
     <row r="72" spans="1:12">
       <c r="A72">
-        <v>9.65324396498629</v>
+        <v>8.237750053405762</v>
       </c>
       <c r="B72">
-        <v>9.46876527194159</v>
+        <v>8.16302490234375</v>
       </c>
       <c r="C72">
-        <v>7.606774087745229</v>
+        <v>7.495575428009033</v>
       </c>
       <c r="D72">
-        <v>7.141370130163642</v>
+        <v>6.958286285400391</v>
       </c>
       <c r="E72">
-        <v>6.619332198718535</v>
+        <v>7.734150886535645</v>
       </c>
       <c r="F72">
-        <v>5.385873227632236</v>
+        <v>5.077700614929199</v>
       </c>
       <c r="G72">
-        <v>6.40308345944083</v>
+        <v>7.501604557037354</v>
       </c>
       <c r="H72">
-        <v>12.00040193982425</v>
+        <v>13.1417760848999</v>
       </c>
       <c r="I72">
-        <v>12.12702943818972</v>
+        <v>8.73421573638916</v>
       </c>
       <c r="J72">
-        <v>12.8728444796219</v>
+        <v>9.885271072387695</v>
       </c>
       <c r="K72">
-        <v>12.88121707719058</v>
+        <v>11.15431976318359</v>
       </c>
       <c r="L72" t="s">
         <v>229</v>
@@ -83744,37 +83744,37 @@
     </row>
     <row r="73" spans="1:12">
       <c r="A73">
-        <v>9.482485722206469</v>
+        <v>8.226492881774902</v>
       </c>
       <c r="B73">
-        <v>9.59816940811131</v>
+        <v>8.150839805603027</v>
       </c>
       <c r="C73">
-        <v>7.538790644902411</v>
+        <v>7.492869853973389</v>
       </c>
       <c r="D73">
-        <v>7.160627960392035</v>
+        <v>6.951699733734131</v>
       </c>
       <c r="E73">
-        <v>6.481236795718693</v>
+        <v>7.744112968444824</v>
       </c>
       <c r="F73">
-        <v>5.364692343749786</v>
+        <v>5.062688827514648</v>
       </c>
       <c r="G73">
-        <v>6.260454462962705</v>
+        <v>7.503138542175293</v>
       </c>
       <c r="H73">
-        <v>11.92242833632964</v>
+        <v>13.12636089324951</v>
       </c>
       <c r="I73">
-        <v>11.70748662791568</v>
+        <v>8.73207950592041</v>
       </c>
       <c r="J73">
-        <v>12.50221466401073</v>
+        <v>9.869697570800781</v>
       </c>
       <c r="K73">
-        <v>12.76275397214235</v>
+        <v>11.13765716552734</v>
       </c>
       <c r="L73" t="s">
         <v>229</v>
@@ -83782,37 +83782,37 @@
     </row>
     <row r="74" spans="1:12">
       <c r="A74">
-        <v>9.327135275145979</v>
+        <v>8.200832366943359</v>
       </c>
       <c r="B74">
-        <v>9.562873440177757</v>
+        <v>8.092103004455566</v>
       </c>
       <c r="C74">
-        <v>7.607326232859867</v>
+        <v>7.477029800415039</v>
       </c>
       <c r="D74">
-        <v>7.335961794793313</v>
+        <v>6.944353103637695</v>
       </c>
       <c r="E74">
-        <v>5.648582964440528</v>
+        <v>7.740015983581543</v>
       </c>
       <c r="F74">
-        <v>5.385873227632236</v>
+        <v>5.030267238616943</v>
       </c>
       <c r="G74">
-        <v>6.088456897128902</v>
+        <v>7.512514591217041</v>
       </c>
       <c r="H74">
-        <v>11.87151402138413</v>
+        <v>13.07465648651123</v>
       </c>
       <c r="I74">
-        <v>11.30453368181164</v>
+        <v>8.7208251953125</v>
       </c>
       <c r="J74">
-        <v>11.77988598889701</v>
+        <v>9.846271514892578</v>
       </c>
       <c r="K74">
-        <v>12.44411356595004</v>
+        <v>11.12046241760254</v>
       </c>
       <c r="L74" t="s">
         <v>229</v>
@@ -83820,37 +83820,37 @@
     </row>
     <row r="75" spans="1:12">
       <c r="A75">
-        <v>9.591436896657521</v>
+        <v>8.191437721252441</v>
       </c>
       <c r="B75">
-        <v>9.544746976647914</v>
+        <v>8.092922210693359</v>
       </c>
       <c r="C75">
-        <v>7.640443650183121</v>
+        <v>7.474401473999023</v>
       </c>
       <c r="D75">
-        <v>7.287952564361452</v>
+        <v>6.956449031829834</v>
       </c>
       <c r="E75">
-        <v>5.910495514694796</v>
+        <v>7.725958347320557</v>
       </c>
       <c r="F75">
-        <v>5.765047629465196</v>
+        <v>5.018047332763672</v>
       </c>
       <c r="G75">
-        <v>6.23416864848976</v>
+        <v>7.505778312683105</v>
       </c>
       <c r="H75">
-        <v>11.8387996768227</v>
+        <v>13.10097599029541</v>
       </c>
       <c r="I75">
-        <v>11.74588732258116</v>
+        <v>8.699663162231445</v>
       </c>
       <c r="J75">
-        <v>12.11261019961371</v>
+        <v>9.841140747070312</v>
       </c>
       <c r="K75">
-        <v>12.55020199860994</v>
+        <v>11.10415649414062</v>
       </c>
       <c r="L75" t="s">
         <v>229</v>
@@ -83858,37 +83858,37 @@
     </row>
     <row r="76" spans="1:12">
       <c r="A76">
-        <v>9.511678795536362</v>
+        <v>8.181634902954102</v>
       </c>
       <c r="B76">
-        <v>9.492283784773306</v>
+        <v>8.07929801940918</v>
       </c>
       <c r="C76">
-        <v>7.597897950521784</v>
+        <v>7.472992420196533</v>
       </c>
       <c r="D76">
-        <v>7.295520809990901</v>
+        <v>6.95713472366333</v>
       </c>
       <c r="E76">
-        <v>5.734778592978486</v>
+        <v>7.721131801605225</v>
       </c>
       <c r="F76">
-        <v>5.631516184147461</v>
+        <v>5.018177509307861</v>
       </c>
       <c r="G76">
-        <v>6.207173194561537</v>
+        <v>7.50537633895874</v>
       </c>
       <c r="H76">
-        <v>11.81321275665597</v>
+        <v>13.07718753814697</v>
       </c>
       <c r="I76">
-        <v>11.27014593347344</v>
+        <v>8.707076072692871</v>
       </c>
       <c r="J76">
-        <v>11.84294039081997</v>
+        <v>9.83692741394043</v>
       </c>
       <c r="K76">
-        <v>12.44222893867714</v>
+        <v>11.10195350646973</v>
       </c>
       <c r="L76" t="s">
         <v>229</v>
@@ -83896,37 +83896,37 @@
     </row>
     <row r="77" spans="1:12">
       <c r="A77">
-        <v>9.469708691540703</v>
+        <v>8.179313659667969</v>
       </c>
       <c r="B77">
-        <v>9.527095716197303</v>
+        <v>8.076800346374512</v>
       </c>
       <c r="C77">
-        <v>7.526298626007885</v>
+        <v>7.476440906524658</v>
       </c>
       <c r="D77">
-        <v>7.178184103286359</v>
+        <v>6.955240726470947</v>
       </c>
       <c r="E77">
-        <v>5.84515341175989</v>
+        <v>7.714281558990479</v>
       </c>
       <c r="F77">
-        <v>5.361629584612668</v>
+        <v>5.023970127105713</v>
       </c>
       <c r="G77">
-        <v>6.3591893272333</v>
+        <v>7.497026920318604</v>
       </c>
       <c r="H77">
-        <v>11.79671413445553</v>
+        <v>13.0642671585083</v>
       </c>
       <c r="I77">
-        <v>11.45858660069722</v>
+        <v>8.714846611022949</v>
       </c>
       <c r="J77">
-        <v>12.01899982132026</v>
+        <v>9.836307525634766</v>
       </c>
       <c r="K77">
-        <v>12.47689251425009</v>
+        <v>11.10312843322754</v>
       </c>
       <c r="L77" t="s">
         <v>229</v>
@@ -83934,37 +83934,37 @@
     </row>
     <row r="78" spans="1:12">
       <c r="A78">
-        <v>9.523933801851928</v>
+        <v>8.173800468444824</v>
       </c>
       <c r="B78">
-        <v>9.38560005231319</v>
+        <v>8.049766540527344</v>
       </c>
       <c r="C78">
-        <v>7.547032743766312</v>
+        <v>7.466324329376221</v>
       </c>
       <c r="D78">
-        <v>7.233307621266355</v>
+        <v>6.955141544342041</v>
       </c>
       <c r="E78">
-        <v>5.452468117803864</v>
+        <v>7.713261604309082</v>
       </c>
       <c r="F78">
-        <v>5.517531560982196</v>
+        <v>5.007616519927979</v>
       </c>
       <c r="G78">
-        <v>5.934306133268033</v>
+        <v>7.507867813110352</v>
       </c>
       <c r="H78">
-        <v>11.77973028287825</v>
+        <v>13.06900215148926</v>
       </c>
       <c r="I78">
-        <v>11.0524760485293</v>
+        <v>8.708479881286621</v>
       </c>
       <c r="J78">
-        <v>11.75986366485015</v>
+        <v>9.832778930664062</v>
       </c>
       <c r="K78">
-        <v>12.4324863998969</v>
+        <v>11.09310722351074</v>
       </c>
       <c r="L78" t="s">
         <v>229</v>
@@ -83972,37 +83972,37 @@
     </row>
     <row r="79" spans="1:12">
       <c r="A79">
-        <v>9.366869136203658</v>
+        <v>8.176037788391113</v>
       </c>
       <c r="B79">
-        <v>9.407732954838984</v>
+        <v>8.064058303833008</v>
       </c>
       <c r="C79">
-        <v>7.511828374814633</v>
+        <v>7.480287075042725</v>
       </c>
       <c r="D79">
-        <v>7.254616148363338</v>
+        <v>6.956037998199463</v>
       </c>
       <c r="E79">
-        <v>5.564945987248793</v>
+        <v>7.705377101898193</v>
       </c>
       <c r="F79">
-        <v>5.622104443641934</v>
+        <v>5.024653434753418</v>
       </c>
       <c r="G79">
-        <v>6.184530719520789</v>
+        <v>7.503241062164307</v>
       </c>
       <c r="H79">
-        <v>11.76796984200206</v>
+        <v>13.06477069854736</v>
       </c>
       <c r="I79">
-        <v>11.40037870108298</v>
+        <v>8.717074394226074</v>
       </c>
       <c r="J79">
-        <v>11.81137436900613</v>
+        <v>9.833663940429688</v>
       </c>
       <c r="K79">
-        <v>12.39009183552911</v>
+        <v>11.10075378417969</v>
       </c>
       <c r="L79" t="s">
         <v>229</v>
@@ -84010,37 +84010,37 @@
     </row>
     <row r="80" spans="1:12">
       <c r="A80">
-        <v>9.414187825286588</v>
+        <v>8.153536796569824</v>
       </c>
       <c r="B80">
-        <v>9.79031885443049</v>
+        <v>8.04953670501709</v>
       </c>
       <c r="C80">
-        <v>7.49034328759006</v>
+        <v>7.481612682342529</v>
       </c>
       <c r="D80">
-        <v>7.163801814797807</v>
+        <v>6.969230175018311</v>
       </c>
       <c r="E80">
-        <v>5.63677174457126</v>
+        <v>7.693918704986572</v>
       </c>
       <c r="F80">
-        <v>5.449663107807231</v>
+        <v>5.022510528564453</v>
       </c>
       <c r="G80">
-        <v>6.505986995854929</v>
+        <v>7.488848209381104</v>
       </c>
       <c r="H80">
-        <v>11.75525445982857</v>
+        <v>13.0409517288208</v>
       </c>
       <c r="I80">
-        <v>11.2035278271223</v>
+        <v>8.724053382873535</v>
       </c>
       <c r="J80">
-        <v>11.8322596156784</v>
+        <v>9.825881958007812</v>
       </c>
       <c r="K80">
-        <v>12.38661947843289</v>
+        <v>11.09297561645508</v>
       </c>
       <c r="L80" t="s">
         <v>229</v>
@@ -84048,37 +84048,37 @@
     </row>
     <row r="81" spans="1:12">
       <c r="A81">
-        <v>9.481638990590399</v>
+        <v>8.149126052856445</v>
       </c>
       <c r="B81">
-        <v>9.507477603198719</v>
+        <v>8.034111976623535</v>
       </c>
       <c r="C81">
-        <v>7.497145601781739</v>
+        <v>7.486312389373779</v>
       </c>
       <c r="D81">
-        <v>7.122678016019414</v>
+        <v>6.961596965789795</v>
       </c>
       <c r="E81">
-        <v>5.656380196926665</v>
+        <v>7.668915271759033</v>
       </c>
       <c r="F81">
-        <v>5.517531560982196</v>
+        <v>5.023788928985596</v>
       </c>
       <c r="G81">
-        <v>6.5278857902651</v>
+        <v>7.479886531829834</v>
       </c>
       <c r="H81">
-        <v>11.74488074551336</v>
+        <v>13.03565311431885</v>
       </c>
       <c r="I81">
-        <v>11.57829697657489</v>
+        <v>8.723251342773438</v>
       </c>
       <c r="J81">
-        <v>12.02507687748979</v>
+        <v>9.81904411315918</v>
       </c>
       <c r="K81">
-        <v>12.47629908349221</v>
+        <v>11.08304786682129</v>
       </c>
       <c r="L81" t="s">
         <v>229</v>
@@ -84086,37 +84086,37 @@
     </row>
     <row r="82" spans="1:12">
       <c r="A82">
-        <v>10.19756580077335</v>
+        <v>9.107653617858887</v>
       </c>
       <c r="B82">
-        <v>8.828754570204747</v>
+        <v>6.990021228790283</v>
       </c>
       <c r="C82">
-        <v>5.789960170897253</v>
+        <v>7.236083507537842</v>
       </c>
       <c r="D82">
-        <v>3.697613568865205</v>
+        <v>5.231846332550049</v>
       </c>
       <c r="E82">
-        <v>5.438079308923196</v>
+        <v>7.074573993682861</v>
       </c>
       <c r="F82">
-        <v>4.336906199393412</v>
+        <v>5.759976863861084</v>
       </c>
       <c r="G82">
-        <v>8.14544937540464</v>
+        <v>10.2762622833252</v>
       </c>
       <c r="H82">
-        <v>10.8106298982435</v>
+        <v>13.07784843444824</v>
       </c>
       <c r="I82">
-        <v>9.054595855999962</v>
+        <v>8.409500122070312</v>
       </c>
       <c r="J82">
-        <v>12.05459708936681</v>
+        <v>11.71580505371094</v>
       </c>
       <c r="K82">
-        <v>12.04833312350577</v>
+        <v>11.97125053405762</v>
       </c>
       <c r="L82" t="s">
         <v>230</v>
@@ -84124,37 +84124,37 @@
     </row>
     <row r="83" spans="1:12">
       <c r="A83">
-        <v>10.20622242350979</v>
+        <v>9.171847343444824</v>
       </c>
       <c r="B83">
-        <v>8.828754570204747</v>
+        <v>7.063360691070557</v>
       </c>
       <c r="C83">
-        <v>5.920386288426155</v>
+        <v>7.310327529907227</v>
       </c>
       <c r="D83">
-        <v>3.433798731716781</v>
+        <v>5.310366153717041</v>
       </c>
       <c r="E83">
-        <v>5.317575237648362</v>
+        <v>7.229138851165771</v>
       </c>
       <c r="F83">
-        <v>4.821756284124562</v>
+        <v>5.839672088623047</v>
       </c>
       <c r="G83">
-        <v>8.124461468563267</v>
+        <v>10.50975799560547</v>
       </c>
       <c r="H83">
-        <v>10.77007904095346</v>
+        <v>13.18149471282959</v>
       </c>
       <c r="I83">
-        <v>8.983300364325961</v>
+        <v>8.482417106628418</v>
       </c>
       <c r="J83">
-        <v>12.04993202541774</v>
+        <v>11.82016563415527</v>
       </c>
       <c r="K83">
-        <v>12.01432681746944</v>
+        <v>12.04637908935547</v>
       </c>
       <c r="L83" t="s">
         <v>230</v>
@@ -84162,37 +84162,37 @@
     </row>
     <row r="84" spans="1:12">
       <c r="A84">
-        <v>10.26558113410534</v>
+        <v>9.139287948608398</v>
       </c>
       <c r="B84">
-        <v>8.346800284538936</v>
+        <v>7.010001182556152</v>
       </c>
       <c r="C84">
-        <v>5.855708395827875</v>
+        <v>7.238355159759521</v>
       </c>
       <c r="D84">
-        <v>3.523948950376441</v>
+        <v>5.297237873077393</v>
       </c>
       <c r="E84">
-        <v>5.261538230318509</v>
+        <v>7.136418342590332</v>
       </c>
       <c r="F84">
-        <v>4.336906199393412</v>
+        <v>5.762889862060547</v>
       </c>
       <c r="G84">
-        <v>7.965888454154388</v>
+        <v>10.37394523620605</v>
       </c>
       <c r="H84">
-        <v>10.74209778452577</v>
+        <v>13.12178516387939</v>
       </c>
       <c r="I84">
-        <v>9.067495918541654</v>
+        <v>8.397666931152344</v>
       </c>
       <c r="J84">
-        <v>11.95016912990554</v>
+        <v>11.7806339263916</v>
       </c>
       <c r="K84">
-        <v>11.9706526587028</v>
+        <v>12.02371788024902</v>
       </c>
       <c r="L84" t="s">
         <v>230</v>
@@ -84200,37 +84200,37 @@
     </row>
     <row r="85" spans="1:12">
       <c r="A85">
-        <v>10.37084881881367</v>
+        <v>9.04533576965332</v>
       </c>
       <c r="B85">
-        <v>8.950417554749455</v>
+        <v>6.983511447906494</v>
       </c>
       <c r="C85">
-        <v>5.8001021447537</v>
+        <v>7.192633628845215</v>
       </c>
       <c r="D85">
-        <v>3.523948950376441</v>
+        <v>5.150025844573975</v>
       </c>
       <c r="E85">
-        <v>5.275844482286887</v>
+        <v>6.970448017120361</v>
       </c>
       <c r="F85">
-        <v>3.82322779235926</v>
+        <v>5.719632625579834</v>
       </c>
       <c r="G85">
-        <v>7.927003641897808</v>
+        <v>10.0129508972168</v>
       </c>
       <c r="H85">
-        <v>10.72668054375652</v>
+        <v>13.02816295623779</v>
       </c>
       <c r="I85">
-        <v>8.979108699818939</v>
+        <v>8.341799736022949</v>
       </c>
       <c r="J85">
-        <v>11.99822129520766</v>
+        <v>11.6250057220459</v>
       </c>
       <c r="K85">
-        <v>11.95663502779516</v>
+        <v>11.90442848205566</v>
       </c>
       <c r="L85" t="s">
         <v>230</v>
@@ -84238,37 +84238,37 @@
     </row>
     <row r="86" spans="1:12">
       <c r="A86">
-        <v>10.27750021091688</v>
+        <v>9.051982879638672</v>
       </c>
       <c r="B86">
-        <v>9.239899174217728</v>
+        <v>6.960287570953369</v>
       </c>
       <c r="C86">
-        <v>5.902329735407591</v>
+        <v>7.15706205368042</v>
       </c>
       <c r="D86">
-        <v>3.506557371004054</v>
+        <v>5.150568962097168</v>
       </c>
       <c r="E86">
-        <v>5.014332119077212</v>
+        <v>6.992008686065674</v>
       </c>
       <c r="F86">
-        <v>4.418919272314087</v>
+        <v>5.69064998626709</v>
       </c>
       <c r="G86">
-        <v>8.023342016410552</v>
+        <v>10.05411529541016</v>
       </c>
       <c r="H86">
-        <v>10.70864061978348</v>
+        <v>13.02503681182861</v>
       </c>
       <c r="I86">
-        <v>9.197142562768599</v>
+        <v>8.32420539855957</v>
       </c>
       <c r="J86">
-        <v>12.03652910109543</v>
+        <v>11.63168144226074</v>
       </c>
       <c r="K86">
-        <v>12.02816134723357</v>
+        <v>11.89385032653809</v>
       </c>
       <c r="L86" t="s">
         <v>230</v>
@@ -84276,37 +84276,37 @@
     </row>
     <row r="87" spans="1:12">
       <c r="A87">
-        <v>9.982709415716675</v>
+        <v>9.094736099243164</v>
       </c>
       <c r="B87">
-        <v>8.321448587263115</v>
+        <v>6.966202735900879</v>
       </c>
       <c r="C87">
-        <v>5.755390569488892</v>
+        <v>7.161714553833008</v>
       </c>
       <c r="D87">
-        <v>3.48885796307766</v>
+        <v>5.194710254669189</v>
       </c>
       <c r="E87">
-        <v>4.925642242553173</v>
+        <v>7.078381061553955</v>
       </c>
       <c r="F87">
-        <v>4.362223757377671</v>
+        <v>5.678746700286865</v>
       </c>
       <c r="G87">
-        <v>8.014809206911632</v>
+        <v>10.2293872833252</v>
       </c>
       <c r="H87">
-        <v>10.69208884231479</v>
+        <v>13.06116771697998</v>
       </c>
       <c r="I87">
-        <v>8.818449416779055</v>
+        <v>8.33488941192627</v>
       </c>
       <c r="J87">
-        <v>11.97336265010635</v>
+        <v>11.72585868835449</v>
       </c>
       <c r="K87">
-        <v>11.86188292861858</v>
+        <v>11.96931648254395</v>
       </c>
       <c r="L87" t="s">
         <v>230</v>
@@ -84314,37 +84314,37 @@
     </row>
     <row r="88" spans="1:12">
       <c r="A88">
-        <v>10.32890050615397</v>
+        <v>9.041504859924316</v>
       </c>
       <c r="B88">
-        <v>8.865499838625629</v>
+        <v>6.934070110321045</v>
       </c>
       <c r="C88">
-        <v>5.826655349889321</v>
+        <v>7.177606582641602</v>
       </c>
       <c r="D88">
-        <v>3.697613568865205</v>
+        <v>5.155803203582764</v>
       </c>
       <c r="E88">
-        <v>5.244095841706911</v>
+        <v>7.019275665283203</v>
       </c>
       <c r="F88">
-        <v>4.378753637197711</v>
+        <v>5.693586349487305</v>
       </c>
       <c r="G88">
-        <v>7.994195003910021</v>
+        <v>10.12643241882324</v>
       </c>
       <c r="H88">
-        <v>10.68131283417586</v>
+        <v>13.015212059021</v>
       </c>
       <c r="I88">
-        <v>8.885225555002142</v>
+        <v>8.336577415466309</v>
       </c>
       <c r="J88">
-        <v>11.99004951499465</v>
+        <v>11.66011810302734</v>
       </c>
       <c r="K88">
-        <v>11.96118750572388</v>
+        <v>11.90393447875977</v>
       </c>
       <c r="L88" t="s">
         <v>230</v>
@@ -84352,37 +84352,37 @@
     </row>
     <row r="89" spans="1:12">
       <c r="A89">
-        <v>9.955130785687967</v>
+        <v>9.071452140808105</v>
       </c>
       <c r="B89">
-        <v>8.767519442722172</v>
+        <v>6.966516971588135</v>
       </c>
       <c r="C89">
-        <v>5.71958298651425</v>
+        <v>7.170230865478516</v>
       </c>
       <c r="D89">
-        <v>3.506557371004054</v>
+        <v>5.147569179534912</v>
       </c>
       <c r="E89">
-        <v>5.115995709754077</v>
+        <v>7.021216869354248</v>
       </c>
       <c r="F89">
-        <v>4.169852114730245</v>
+        <v>5.679747104644775</v>
       </c>
       <c r="G89">
-        <v>7.990020682393433</v>
+        <v>10.12733459472656</v>
       </c>
       <c r="H89">
-        <v>10.66432453412203</v>
+        <v>13.01931190490723</v>
       </c>
       <c r="I89">
-        <v>8.871286967004236</v>
+        <v>8.346781730651855</v>
       </c>
       <c r="J89">
-        <v>11.92818687886899</v>
+        <v>11.65643119812012</v>
       </c>
       <c r="K89">
-        <v>11.91045546656262</v>
+        <v>11.92122268676758</v>
       </c>
       <c r="L89" t="s">
         <v>230</v>
@@ -84390,37 +84390,37 @@
     </row>
     <row r="90" spans="1:12">
       <c r="A90">
-        <v>10.37674974190345</v>
+        <v>9.065959930419922</v>
       </c>
       <c r="B90">
-        <v>8.640393703787852</v>
+        <v>6.942018985748291</v>
       </c>
       <c r="C90">
-        <v>5.74833095718719</v>
+        <v>7.150513172149658</v>
       </c>
       <c r="D90">
-        <v>3.48885796307766</v>
+        <v>5.14711332321167</v>
       </c>
       <c r="E90">
-        <v>5.064702620629684</v>
+        <v>7.007619380950928</v>
       </c>
       <c r="F90">
-        <v>4.256863491719876</v>
+        <v>5.667993545532227</v>
       </c>
       <c r="G90">
-        <v>8.116752473228095</v>
+        <v>10.09323692321777</v>
       </c>
       <c r="H90">
-        <v>10.65383388645338</v>
+        <v>13.02995014190674</v>
       </c>
       <c r="I90">
-        <v>8.980507874457484</v>
+        <v>8.337529182434082</v>
       </c>
       <c r="J90">
-        <v>11.98313046144022</v>
+        <v>11.67267799377441</v>
       </c>
       <c r="K90">
-        <v>11.92616031034275</v>
+        <v>11.91396141052246</v>
       </c>
       <c r="L90" t="s">
         <v>230</v>
@@ -84428,37 +84428,37 @@
     </row>
     <row r="91" spans="1:12">
       <c r="A91">
-        <v>9.789073846807304</v>
+        <v>9.062797546386719</v>
       </c>
       <c r="B91">
-        <v>8.677041949176314</v>
+        <v>6.985880374908447</v>
       </c>
       <c r="C91">
-        <v>5.765887412029423</v>
+        <v>7.158109188079834</v>
       </c>
       <c r="D91">
-        <v>3.292147808583199</v>
+        <v>5.142504215240479</v>
       </c>
       <c r="E91">
-        <v>4.980557800691038</v>
+        <v>7.0285964012146</v>
       </c>
       <c r="F91">
-        <v>4.219123548352339</v>
+        <v>5.646488189697266</v>
       </c>
       <c r="G91">
-        <v>7.962884280400202</v>
+        <v>10.11863136291504</v>
       </c>
       <c r="H91">
-        <v>10.64324527480381</v>
+        <v>13.01948642730713</v>
       </c>
       <c r="I91">
-        <v>8.558974661492572</v>
+        <v>8.323502540588379</v>
       </c>
       <c r="J91">
-        <v>11.95282062418475</v>
+        <v>11.63578796386719</v>
       </c>
       <c r="K91">
-        <v>11.88236415858328</v>
+        <v>11.92133331298828</v>
       </c>
       <c r="L91" t="s">
         <v>230</v>

</xml_diff>